<commit_message>
UK rental: rebuild tax tabs with formulas, add Swedish capital tax calc, fix 2025 FX rate to 12.92163
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AY16"/>
+  <dimension ref="B1:AY16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="22.1640625" bestFit="1" customWidth="1" style="4" min="2" max="2"/>
@@ -4336,12 +4336,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" style="4" min="1" max="1"/>
-    <col width="13" customWidth="1" style="4" min="2" max="2"/>
-    <col width="14" customWidth="1" style="4" min="3" max="3"/>
+    <col width="62" customWidth="1" style="4" min="1" max="1"/>
+    <col width="14" customWidth="1" style="4" min="2" max="2"/>
+    <col width="15" customWidth="1" style="4" min="3" max="3"/>
+    <col width="30" customWidth="1" style="4" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4352,406 +4353,626 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Parameters (edit these to recalc):</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>FX rate (SEK per GBP)</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B4" t="n">
         <v>13.50453</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Riksbanken 2024 annual avg</t>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Riksbanken 2024 annual average</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>UK tax year 24/25 (6 April to 5 April)</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>UK tax year (label/float)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>24/25</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>GBP</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Swedish tax year</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2024</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rental Income</t>
+          <t>UK personal allowance</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29925.82</v>
+        <v>12570</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Knight Frank Commission (mgmt + letting)</t>
+          <t>UK basic rate</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-4859.64</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Net Income before Expenses</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>25066.18</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UK financing-cost credit rate</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Repair and Maintenance Expenses</t>
+          <t>Swedish standard deduction (SEK)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-2124.99</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Taxable Property Profit (SA105 box 38/40)</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="n">
-        <v>22941.19</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Memo — residential property finance costs (SA105 box 44):</t>
-        </is>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Swedish % deduction (of rental income)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Swedish capital income tax rate</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Mortgage interest</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>3161.82</v>
-      </c>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>UK tax year 24/25 (6 April to 5 April)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Mortgage product fees</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1749</v>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Total residential finance costs</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>4910.82</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rental Income</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>SUMIF('76A Ingelow Road'!$C$2:$AY$2,$B$5,'76A Ingelow Road'!$C$6:$AY$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Knight Frank Commission (mgmt + letting)</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>SUMIF('76A Ingelow Road'!$C$2:$AY$2,$B$5,'76A Ingelow Road'!$C$10:$AY$10)+SUMIF('76A Ingelow Road'!$C$2:$AY$2,$B$5,'76A Ingelow Road'!$C$11:$AY$11)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>UK tax calculation</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="14" t="n"/>
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Net Income before Expenses</t>
+        </is>
+      </c>
+      <c r="B18" s="12">
+        <f>$B$16+$B$17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Personal Allowance (0%)</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>12570</v>
+          <t>Repair and Maintenance Expenses</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>SUMIF('76A Ingelow Road'!$C$2:$AY$2,$B$5,'76A Ingelow Road'!$C$13:$AY$13)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Basic rate band cap (20% to £50,270)</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>50270</v>
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Taxable Property Profit (SA105 box 38/40)</t>
+        </is>
+      </c>
+      <c r="B20" s="15">
+        <f>$B$18+$B$19</f>
+        <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Total taxable income (property profit)</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>22941.19</v>
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Memo — residential property finance costs (SA105 box 44):</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Above personal allowance</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>10371.19</v>
+          <t xml:space="preserve">  Mortgage interest</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>SUMIF('Santander'!$B$3:$AN$3,$C$5,'Santander'!$B$6:$AN$6)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Basic rate tax (20%)</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>2074.24</v>
+          <t xml:space="preserve">  Mortgage product fees</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>SUMIF('Santander'!$B$3:$AN$3,$C$5,'Santander'!$B$8:$AN$8)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Less: financing cost credit (20% × £4,910.82)</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>-982.16</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Net UK Tax</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="n">
-        <v>1092.08</v>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total residential finance costs</t>
+        </is>
+      </c>
+      <c r="B25" s="12">
+        <f>$B$23+$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>UK tax calculation</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n"/>
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="14" t="n"/>
+      <c r="E27" s="14" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Total taxable income (property profit)</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>$B$20</f>
+        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>Swedish tax year 2024 (1 January to 31 December)</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Above personal allowance</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>MAX(0,$B$20-$B$7)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>SEK</t>
-        </is>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Basic rate tax (= above PA × basic rate)</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>$B$29*$B$8</f>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Rental Income</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>29406.82</v>
-      </c>
-      <c r="C31" t="n">
-        <v>397125.28</v>
+          <t>Less: financing cost credit (finance costs × credit rate)</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>-$B$25*$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Knight Frank Commission</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>-4833.24</v>
-      </c>
-      <c r="C32" t="n">
-        <v>-65270.63</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t>Rental income net of commission (basis for schablonavdrag)</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n">
-        <v>24573.58</v>
-      </c>
-      <c r="C33" s="15" t="n">
-        <v>331854.65</v>
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Net UK Tax</t>
+        </is>
+      </c>
+      <c r="B32" s="17">
+        <f>$B$30+$B$31</f>
+        <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>Schablonavdrag (replaces actual expense deduction):</t>
-        </is>
-      </c>
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Swedish tax year 2024 (1 January to 31 December)</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Standard SEK 40,000 deduction</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>-2961.97</v>
-      </c>
-      <c r="C36" t="n">
-        <v>-40000</v>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  20% of rental income (net of commission) deduction</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>-4914.72</v>
-      </c>
-      <c r="C37" t="n">
-        <v>-66370.98</v>
+          <t>Rental Income</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>SUMIF('76A Ingelow Road'!$C$1:$AY$1,$B$6,'76A Ingelow Road'!$C$6:$AY$6)</f>
+        <v/>
+      </c>
+      <c r="C37">
+        <f>B37*$B$4</f>
+        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="inlineStr">
-        <is>
-          <t>Box 7.3 — Överskott vid uthyrning av privatbostad</t>
-        </is>
-      </c>
-      <c r="B38" s="17" t="n">
-        <v>16696.89</v>
-      </c>
-      <c r="C38" s="17" t="n">
-        <v>225483.65</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>Memo — repairs not deductible under schablonavdrag: £-1,677.00</t>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Knight Frank Commission</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>SUMIF('76A Ingelow Road'!$C$1:$AY$1,$B$6,'76A Ingelow Road'!$C$10:$AY$10)+SUMIF('76A Ingelow Road'!$C$1:$AY$1,$B$6,'76A Ingelow Road'!$C$11:$AY$11)</f>
+        <v/>
+      </c>
+      <c r="C38">
+        <f>B38*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Rental income net of commission (basis for schablonavdrag)</t>
+        </is>
+      </c>
+      <c r="B39" s="15">
+        <f>$B$37+$B$38</f>
+        <v/>
+      </c>
+      <c r="C39" s="15">
+        <f>B39*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Schablonavdrag (replaces actual expense deduction):</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>Box 8.1 — Ränteutgifter (mortgage interest)</t>
-        </is>
-      </c>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="14" t="n"/>
-      <c r="D42" s="14" t="n"/>
-      <c r="E42" s="14" t="n"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Standard SEK 40,000 deduction</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>-$B$10/$B$4</f>
+        <v/>
+      </c>
+      <c r="C42">
+        <f>-$B$10</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mortgage interest (calendar year)</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>2803.66</v>
-      </c>
-      <c r="C43" t="n">
-        <v>37862.11</v>
+          <t xml:space="preserve">  20% of rental income (net of commission)</t>
+        </is>
+      </c>
+      <c r="B43">
+        <f>-$B$39*$B$11</f>
+        <v/>
+      </c>
+      <c r="C43">
+        <f>B43*$B$4</f>
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
+          <t>Box 7.3 — Överskott vid uthyrning av privatbostad</t>
+        </is>
+      </c>
+      <c r="B44" s="17">
+        <f>$B$39+$B$42+$B$43</f>
+        <v/>
+      </c>
+      <c r="C44" s="17">
+        <f>B44*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>Memo — repairs (not deductible under schablonavdrag):</t>
+        </is>
+      </c>
+      <c r="B46" s="16">
+        <f>SUMIF('76A Ingelow Road'!$C$1:$AY$1,$B$6,'76A Ingelow Road'!$C$13:$AY$13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>Box 8.1 — Ränteutgifter (mortgage interest + fees)</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="14" t="n"/>
+      <c r="E48" s="14" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Mortgage interest (calendar year)</t>
+        </is>
+      </c>
+      <c r="B49">
+        <f>SUMIF('Santander'!$B$4:$AN$4,$C$6,'Santander'!$B$6:$AN$6)</f>
+        <v/>
+      </c>
+      <c r="C49">
+        <f>B49*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Mortgage product fees (deductible)</t>
+        </is>
+      </c>
+      <c r="B50">
+        <f>SUMIF('Santander'!$B$4:$AN$4,$C$6,'Santander'!$B$8:$AN$8)</f>
+        <v/>
+      </c>
+      <c r="C50">
+        <f>B50*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
           <t>Box 8.1 total</t>
         </is>
       </c>
-      <c r="B44" s="17" t="n">
-        <v>2803.66</v>
-      </c>
-      <c r="C44" s="17" t="n">
-        <v>37862.11</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="B51" s="17">
+        <f>$B$49+$B$50</f>
+        <v/>
+      </c>
+      <c r="C51" s="17">
+        <f>B51*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>Foreign tax credit (Avräkning utländsk skatt)</t>
         </is>
       </c>
-      <c r="B46" s="14" t="n"/>
-      <c r="C46" s="14" t="n"/>
-      <c r="D46" s="14" t="n"/>
-      <c r="E46" s="14" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>UK 23/24 tax × 3/12 (Jan-Mar fell in old UK year)</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>282</v>
-      </c>
-      <c r="C47" t="n">
-        <v>3808.28</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>UK 24/25 tax × 9/12 (Apr-Dec fell in new UK year)</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>819.0599999999999</v>
-      </c>
-      <c r="C48" t="n">
-        <v>11061.02</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="12" t="inlineStr">
-        <is>
-          <t>Apportioned FTC for this Swedish year</t>
-        </is>
-      </c>
-      <c r="B49" s="17" t="n">
-        <v>1101.06</v>
-      </c>
-      <c r="C49" s="17" t="n">
-        <v>14869.3</v>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="14" t="n"/>
+      <c r="E53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>UK prior year tax × 3/12 (Jan-Mar fell in old UK year)</t>
+        </is>
+      </c>
+      <c r="B54">
+        <f>1128*3/12</f>
+        <v/>
+      </c>
+      <c r="C54">
+        <f>B54*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>UK current year tax × 9/12 (Apr-Dec)</t>
+        </is>
+      </c>
+      <c r="B55">
+        <f>$B$32*9/12</f>
+        <v/>
+      </c>
+      <c r="C55">
+        <f>B55*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>Apportioned FTC for Swedish 2024</t>
+        </is>
+      </c>
+      <c r="B56" s="17">
+        <f>1128*3/12+$B$32*9/12</f>
+        <v/>
+      </c>
+      <c r="C56" s="17">
+        <f>B56*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>Swedish tax payable on rental property (marginal calc)</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="14" t="n"/>
+      <c r="E59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t>Note: capital income (rental, interest, dividends) is taxed at flat 30% in Sweden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>Other income (salary ~800,000 SEK) is in earned income (~50% marginal); does not affect this calc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Net capital income (Box 7.3 - Box 8.1)</t>
+        </is>
+      </c>
+      <c r="B63">
+        <f>$B$44-$B$51</f>
+        <v/>
+      </c>
+      <c r="C63">
+        <f>B63*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Capital tax @ 30% (gross, before foreign tax credit)</t>
+        </is>
+      </c>
+      <c r="B64">
+        <f>$B$63*$B$12</f>
+        <v/>
+      </c>
+      <c r="C64">
+        <f>B64*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Less: Foreign tax credit</t>
+        </is>
+      </c>
+      <c r="B65">
+        <f>-$B$56</f>
+        <v/>
+      </c>
+      <c r="C65">
+        <f>B65*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>Swedish tax payable on this property</t>
+        </is>
+      </c>
+      <c r="B66" s="17">
+        <f>$B$64-$B$56</f>
+        <v/>
+      </c>
+      <c r="C66" s="17">
+        <f>B66*$B$4</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -4768,12 +4989,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" style="4" min="1" max="1"/>
-    <col width="13" customWidth="1" style="4" min="2" max="2"/>
-    <col width="14" customWidth="1" style="4" min="3" max="3"/>
+    <col width="62" customWidth="1" style="4" min="1" max="1"/>
+    <col width="14" customWidth="1" style="4" min="2" max="2"/>
+    <col width="15" customWidth="1" style="4" min="3" max="3"/>
+    <col width="30" customWidth="1" style="4" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4784,419 +5006,626 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Parameters (edit these to recalc):</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>FX rate (SEK per GBP)</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>12.919</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Approx 2025 avg (verify vs Riksbanken)</t>
+      <c r="B4" t="n">
+        <v>12.92163</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Riksbanken 2025 annual average</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>UK tax year 25/26 (6 April to 5 April)</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="n"/>
-      <c r="C5" s="14" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="14" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>UK tax year (label/float)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>25.26</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>GBP</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Swedish tax year</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rental Income</t>
+          <t>UK personal allowance</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>32271.25</v>
+        <v>12570</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Knight Frank Commission (mgmt + letting)</t>
+          <t>UK basic rate</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-2859.41</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Net Income before Expenses</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>29411.84</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UK financing-cost credit rate</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Repair and Maintenance Expenses</t>
+          <t>Swedish standard deduction (SEK)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-7942.6</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Taxable Property Profit (SA105 box 38/40)</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="n">
-        <v>21469.24</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Memo — residential property finance costs (SA105 box 44):</t>
-        </is>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Swedish % deduction (of rental income)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Swedish capital income tax rate</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Mortgage interest</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>7829.88</v>
-      </c>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>UK tax year 25/26 (6 April to 5 April)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Mortgage product fees</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0</v>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Total residential finance costs</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="n">
-        <v>7829.88</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rental Income</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>SUMIF('76A Ingelow Road'!$C$2:$AY$2,$B$5,'76A Ingelow Road'!$C$6:$AY$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Knight Frank Commission (mgmt + letting)</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>SUMIF('76A Ingelow Road'!$C$2:$AY$2,$B$5,'76A Ingelow Road'!$C$10:$AY$10)+SUMIF('76A Ingelow Road'!$C$2:$AY$2,$B$5,'76A Ingelow Road'!$C$11:$AY$11)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>UK tax calculation</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="14" t="n"/>
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Net Income before Expenses</t>
+        </is>
+      </c>
+      <c r="B18" s="12">
+        <f>$B$16+$B$17</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Personal Allowance (0%)</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>12570</v>
+          <t>Repair and Maintenance Expenses</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>SUMIF('76A Ingelow Road'!$C$2:$AY$2,$B$5,'76A Ingelow Road'!$C$13:$AY$13)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Basic rate band cap (20% to £50,270)</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>50270</v>
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Taxable Property Profit (SA105 box 38/40)</t>
+        </is>
+      </c>
+      <c r="B20" s="15">
+        <f>$B$18+$B$19</f>
+        <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Total taxable income (property profit)</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>21469.24</v>
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Memo — residential property finance costs (SA105 box 44):</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Above personal allowance</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>8899.24</v>
+          <t xml:space="preserve">  Mortgage interest</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>SUMIF('Santander'!$B$3:$AN$3,$C$5,'Santander'!$B$6:$AN$6)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Basic rate tax (20%)</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1779.85</v>
+          <t xml:space="preserve">  Mortgage product fees</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>SUMIF('Santander'!$B$3:$AN$3,$C$5,'Santander'!$B$8:$AN$8)</f>
+        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Less: financing cost credit (20% × £7,829.88)</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>-1565.98</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Net UK Tax</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="n">
-        <v>213.87</v>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Total residential finance costs</t>
+        </is>
+      </c>
+      <c r="B25" s="12">
+        <f>$B$23+$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>UK tax calculation</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n"/>
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="14" t="n"/>
+      <c r="E27" s="14" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Total taxable income (property profit)</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>$B$20</f>
+        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>Swedish tax year 2025 (1 January to 31 December)</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Above personal allowance</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>MAX(0,$B$20-$B$7)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>SEK</t>
-        </is>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Basic rate tax (= above PA × basic rate)</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>$B$29*$B$8</f>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Rental Income</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>33900</v>
-      </c>
-      <c r="C31" t="n">
-        <v>437954.1</v>
+          <t>Less: financing cost credit (finance costs × credit rate)</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>-$B$25*$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Knight Frank Commission</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>-5061.6</v>
-      </c>
-      <c r="C32" t="n">
-        <v>-65390.81</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t>Rental income net of commission (basis for schablonavdrag)</t>
-        </is>
-      </c>
-      <c r="B33" s="15" t="n">
-        <v>28838.4</v>
-      </c>
-      <c r="C33" s="15" t="n">
-        <v>372563.29</v>
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>Net UK Tax</t>
+        </is>
+      </c>
+      <c r="B32" s="17">
+        <f>$B$30+$B$31</f>
+        <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
-        <is>
-          <t>Schablonavdrag (replaces actual expense deduction):</t>
-        </is>
-      </c>
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Swedish tax year 2025 (1 January to 31 December)</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Standard SEK 40,000 deduction</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>-3096.21</v>
-      </c>
-      <c r="C36" t="n">
-        <v>-40000</v>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  20% of rental income (net of commission) deduction</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>-5767.68</v>
-      </c>
-      <c r="C37" t="n">
-        <v>-74512.66</v>
+          <t>Rental Income</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>SUMIF('76A Ingelow Road'!$C$1:$AY$1,$B$6,'76A Ingelow Road'!$C$6:$AY$6)</f>
+        <v/>
+      </c>
+      <c r="C37">
+        <f>B37*$B$4</f>
+        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="12" t="inlineStr">
-        <is>
-          <t>Box 7.3 — Överskott vid uthyrning av privatbostad</t>
-        </is>
-      </c>
-      <c r="B38" s="17" t="n">
-        <v>19974.51</v>
-      </c>
-      <c r="C38" s="17" t="n">
-        <v>258050.69</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>Memo — repairs not deductible under schablonavdrag: £-3,243.99</t>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Knight Frank Commission</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>SUMIF('76A Ingelow Road'!$C$1:$AY$1,$B$6,'76A Ingelow Road'!$C$10:$AY$10)+SUMIF('76A Ingelow Road'!$C$1:$AY$1,$B$6,'76A Ingelow Road'!$C$11:$AY$11)</f>
+        <v/>
+      </c>
+      <c r="C38">
+        <f>B38*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Rental income net of commission (basis for schablonavdrag)</t>
+        </is>
+      </c>
+      <c r="B39" s="15">
+        <f>$B$37+$B$38</f>
+        <v/>
+      </c>
+      <c r="C39" s="15">
+        <f>B39*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Schablonavdrag (replaces actual expense deduction):</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>Box 8.1 — Ränteutgifter (mortgage interest)</t>
-        </is>
-      </c>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="14" t="n"/>
-      <c r="D42" s="14" t="n"/>
-      <c r="E42" s="14" t="n"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Standard SEK 40,000 deduction</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>-$B$10/$B$4</f>
+        <v/>
+      </c>
+      <c r="C42">
+        <f>-$B$10</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mortgage interest (calendar year)</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>6955.02</v>
-      </c>
-      <c r="C43" t="n">
-        <v>89851.89999999999</v>
+          <t xml:space="preserve">  20% of rental income (net of commission)</t>
+        </is>
+      </c>
+      <c r="B43">
+        <f>-$B$39*$B$11</f>
+        <v/>
+      </c>
+      <c r="C43">
+        <f>B43*$B$4</f>
+        <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Mortgage product fees (also deductible)</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>1749</v>
-      </c>
-      <c r="C44" t="n">
-        <v>22595.33</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t>Box 8.1 total</t>
-        </is>
-      </c>
-      <c r="B45" s="17" t="n">
-        <v>8704.02</v>
-      </c>
-      <c r="C45" s="17" t="n">
-        <v>112447.23</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>Foreign tax credit (Avräkning utländsk skatt)</t>
-        </is>
-      </c>
-      <c r="B47" s="14" t="n"/>
-      <c r="C47" s="14" t="n"/>
-      <c r="D47" s="14" t="n"/>
-      <c r="E47" s="14" t="n"/>
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>Box 7.3 — Överskott vid uthyrning av privatbostad</t>
+        </is>
+      </c>
+      <c r="B44" s="17">
+        <f>$B$39+$B$42+$B$43</f>
+        <v/>
+      </c>
+      <c r="C44" s="17">
+        <f>B44*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>Memo — repairs (not deductible under schablonavdrag):</t>
+        </is>
+      </c>
+      <c r="B46" s="16">
+        <f>SUMIF('76A Ingelow Road'!$C$1:$AY$1,$B$6,'76A Ingelow Road'!$C$13:$AY$13)</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>UK 24/25 tax × 3/12 (Jan-Mar fell in old UK year)</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>273.02</v>
-      </c>
-      <c r="C48" t="n">
-        <v>3527.15</v>
-      </c>
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>Box 8.1 — Ränteutgifter (mortgage interest + fees)</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="14" t="n"/>
+      <c r="E48" s="14" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>UK 25/26 tax × 9/12 (Apr-Dec fell in new UK year)</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>160.4</v>
-      </c>
-      <c r="C49" t="n">
-        <v>2072.24</v>
+          <t>Mortgage interest (calendar year)</t>
+        </is>
+      </c>
+      <c r="B49">
+        <f>SUMIF('Santander'!$B$4:$AN$4,$C$6,'Santander'!$B$6:$AN$6)</f>
+        <v/>
+      </c>
+      <c r="C49">
+        <f>B49*$B$4</f>
+        <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="12" t="inlineStr">
-        <is>
-          <t>Apportioned FTC for this Swedish year</t>
-        </is>
-      </c>
-      <c r="B50" s="17" t="n">
-        <v>433.42</v>
-      </c>
-      <c r="C50" s="17" t="n">
-        <v>5599.35</v>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Mortgage product fees (deductible)</t>
+        </is>
+      </c>
+      <c r="B50">
+        <f>SUMIF('Santander'!$B$4:$AN$4,$C$6,'Santander'!$B$8:$AN$8)</f>
+        <v/>
+      </c>
+      <c r="C50">
+        <f>B50*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>Box 8.1 total</t>
+        </is>
+      </c>
+      <c r="B51" s="17">
+        <f>$B$49+$B$50</f>
+        <v/>
+      </c>
+      <c r="C51" s="17">
+        <f>B51*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>Foreign tax credit (Avräkning utländsk skatt)</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="14" t="n"/>
+      <c r="E53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>UK prior year tax × 3/12 (Jan-Mar fell in old UK year)</t>
+        </is>
+      </c>
+      <c r="B54">
+        <f>'Tax 24-25'!$B$32*3/12</f>
+        <v/>
+      </c>
+      <c r="C54">
+        <f>B54*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>UK current year tax × 9/12 (Apr-Dec)</t>
+        </is>
+      </c>
+      <c r="B55">
+        <f>$B$32*9/12</f>
+        <v/>
+      </c>
+      <c r="C55">
+        <f>B55*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
+        <is>
+          <t>Apportioned FTC for Swedish 2025</t>
+        </is>
+      </c>
+      <c r="B56" s="17">
+        <f>'Tax 24-25'!$B$32*3/12+$B$32*9/12</f>
+        <v/>
+      </c>
+      <c r="C56" s="17">
+        <f>B56*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>Swedish tax payable on rental property (marginal calc)</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="14" t="n"/>
+      <c r="E59" s="14" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
+        <is>
+          <t>Note: capital income (rental, interest, dividends) is taxed at flat 30% in Sweden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>Other income (salary ~800,000 SEK) is in earned income (~50% marginal); does not affect this calc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Net capital income (Box 7.3 - Box 8.1)</t>
+        </is>
+      </c>
+      <c r="B63">
+        <f>$B$44-$B$51</f>
+        <v/>
+      </c>
+      <c r="C63">
+        <f>B63*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Capital tax @ 30% (gross, before foreign tax credit)</t>
+        </is>
+      </c>
+      <c r="B64">
+        <f>$B$63*$B$12</f>
+        <v/>
+      </c>
+      <c r="C64">
+        <f>B64*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Less: Foreign tax credit</t>
+        </is>
+      </c>
+      <c r="B65">
+        <f>-$B$56</f>
+        <v/>
+      </c>
+      <c r="C65">
+        <f>B65*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="12" t="inlineStr">
+        <is>
+          <t>Swedish tax payable on this property</t>
+        </is>
+      </c>
+      <c r="B66" s="17">
+        <f>$B$64-$B$56</f>
+        <v/>
+      </c>
+      <c r="C66" s="17">
+        <f>B66*$B$4</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UK rental: add Capital Gains 2025 tab — Vanguard ISA sold June 2025, ~SEK 34k Swedish tax
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Santander" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Tax 24-25" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Tax 25-26" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Capital Gains 2025" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -5634,4 +5635,372 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" style="4" min="1" max="1"/>
+    <col width="16" customWidth="1" style="4" min="2" max="2"/>
+    <col width="16" customWidth="1" style="4" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Capital Gains 2025 — Vanguard ISA (sold June 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Held in UK ISA → no UK tax. Swedish residency 25 Nov 2021 → cost basis taken at that date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Swedish capital gains tax: 30% flat on net gain in SEK.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Parameters (edit to recalc):</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Cost basis date</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>25 Nov 2021</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>(Swedish tax-residency start)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cost basis value (GBP)</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>23031.31</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cost basis FX rate (Nov 2021)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>11.84728</v>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Riksbanken Nov 2021 monthly avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Sale date</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>5 Jun 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Sale proceeds (GBP)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>29862.97</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Sale FX rate (Jun 2025)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>12.9485</v>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Riksbanken Jun 2025 monthly avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Swedish capital tax rate</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="n"/>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="14" t="n"/>
+      <c r="E15" s="14" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Cost basis (omkostnadsbelopp)</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>$B$8</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>$B$8*$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sale proceeds (försäljningspris)</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>$B$11</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>$B$11*$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Capital gain</t>
+        </is>
+      </c>
+      <c r="B19" s="15">
+        <f>$B$11-$B$8</f>
+        <v/>
+      </c>
+      <c r="C19" s="15">
+        <f>$B$11*$B$12-$B$8*$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Decomposition (memo):</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Investment performance in GBP</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>$B$11-$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FX uplift on cost basis (Nov21 → Jun25)</t>
+        </is>
+      </c>
+      <c r="C23">
+        <f>$B$8*($B$12-$B$9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Total SEK gain (matches above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Swedish capital tax (30% of SEK gain)</t>
+        </is>
+      </c>
+      <c r="B26" s="17">
+        <f>$C$19*$B$13/$B$12</f>
+        <v/>
+      </c>
+      <c r="C26" s="17">
+        <f>$C$19*$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Reporting in your Swedish tax return:</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>• File K4 (bilaga K4) — avsnitt A or C depending on whether marknadsnoterade aktier/fonder</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>• K4 lists: antal/units, försäljningspris, omkostnadsbelopp, vinst</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>• Net gain rolls into Box 7.4 (kapitalvinst marknadsnoterade aktier/fonder) on INK1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>• Box 7.2 catches general interest/dividends; CGT-specific lines are 7.4/7.5/7.6 depending on type</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Assumptions &amp; caveats:</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>• Cost basis taken at 25 Nov 2021 value (Swedish residency start). This is the simplest approach if</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  the bulk of the holding pre-dated the move. If significant contributions were made AFTER Nov 2021,</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Swedish tax law applies the average-cost method (genomsnittsmetoden) — each contribution's own</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  cost basis (in SEK at the time) is weighted into the average. Confirm with accountant if you</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  contributed materially between Nov 2021 and Jun 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>• FX rates used are Riksbanken monthly averages for Nov 2021 and Jun 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>• ISA wrapper provides no Swedish tax benefit — Sweden taxes the gain regardless.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>• Capital losses elsewhere in the same year can offset this gain (currently none assumed).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
UK rental: add HSBC Interest tab (UK 25/26 full ~£242; Swedish 2025 partial pending Jan-Apr statements)
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Tax 24-25" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Tax 25-26" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Capital Gains 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="HSBC Interest" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -71,8 +72,11 @@
     <font>
       <i val="1"/>
     </font>
+    <font>
+      <color rgb="00990000"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -99,6 +103,11 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCCCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -113,7 +122,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +141,10 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6003,4 +6016,681 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="4" min="1" max="1"/>
+    <col width="16" customWidth="1" style="4" min="2" max="2"/>
+    <col width="22" customWidth="1" style="4" min="3" max="3"/>
+    <col width="24" customWidth="1" style="4" min="4" max="4"/>
+    <col width="12" customWidth="1" style="4" min="5" max="5"/>
+    <col width="12" customWidth="1" style="4" min="6" max="6"/>
+    <col width="12" customWidth="1" style="4" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>HSBC Savings Interest — by month credited</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>UK tax: report total in SA100 box 2 (Untaxed UK interest). PSA £1,000 covers basic rate taxpayers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Swedish tax: report in Box 7.2 (Ränteinkomster) — taxed at 30% capital rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Credit date</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>GROSS INTEREST (£)</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>ADDED GROSS INTEREST (£)</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Total (£)</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>UK Tax Year</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Swedish Year</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>01 Jan 25</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>TO 31DEC2024</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>24/25</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>01 Feb 25</t>
+        </is>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>TO 31JAN2025</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>24/25</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>01 Mar 25</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>TO 28FEB2025</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>24/25</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>01 Apr 25</t>
+        </is>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>TO 31MAR2025</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>24/25</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>01 May 25</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TO 30APR2025</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="E11">
+        <f>SUM(C11:D11)</f>
+        <v/>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>01 Jun 25</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TO 31MAY2025</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="E12">
+        <f>SUM(C12:D12)</f>
+        <v/>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>01 Jul 25</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TO 30JUN2025</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="D13" t="n">
+        <v>21.55</v>
+      </c>
+      <c r="E13">
+        <f>SUM(C13:D13)</f>
+        <v/>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>01 Aug 25</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TO 31JUL2025</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="E14">
+        <f>SUM(C14:D14)</f>
+        <v/>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>01 Sep 25</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TO 31AUG2025</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <f>SUM(C15:D15)</f>
+        <v/>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>01 Oct 25</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TO 30SEP2025</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>9.65</v>
+      </c>
+      <c r="D16" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="E16">
+        <f>SUM(C16:D16)</f>
+        <v/>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>01 Nov 25</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TO 31OCT2025</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="D17" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="E17">
+        <f>SUM(C17:D17)</f>
+        <v/>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>01 Dec 25</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TO 30NOV2025</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="D18" t="n">
+        <v>28.62</v>
+      </c>
+      <c r="E18">
+        <f>SUM(C18:D18)</f>
+        <v/>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>01 Jan 26</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TO 31DEC2025</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>11.28</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <f>SUM(C19:D19)</f>
+        <v/>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>01 Feb 26</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TO 31JAN2026</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <f>SUM(C20:D20)</f>
+        <v/>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>01 Mar 26</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>TO 28FEB2026</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <f>SUM(C21:D21)</f>
+        <v/>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>01 Apr 26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TO 31MAR2026</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>6.43</v>
+      </c>
+      <c r="D22" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="E22">
+        <f>SUM(C22:D22)</f>
+        <v/>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>25/26</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Totals by tax year</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="14" t="n"/>
+      <c r="G24" s="14" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr"/>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Total (£)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>UK 25/26 (credits 6 Apr 2025 to 5 Apr 2026)</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>SUMIF(F7:F22,"25/26",E7:E22)</f>
+        <v/>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Full 12 months ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Swedish 2025 (credits Jan-Dec 2025)</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>SUMIF(G7:G22,"2025",E7:E22)</f>
+        <v/>
+      </c>
+      <c r="C27" s="20" t="inlineStr">
+        <is>
+          <t>MISSING Jan-Apr 2025 — partial</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Swedish 2026 partial (Jan-Apr 2026 only)</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>SUMIF(G7:G22,"2026",E7:E22)</f>
+        <v/>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>Will need more data later</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>Notes:</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>• Each month has both a 'GROSS INTEREST TO &lt;date&gt;' line and (sometimes) an 'ADDED GROSS INTEREST' line. Both credit the account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>• UK 25/26 PSA covers £1,000 for basic rate; with ~£240 interest, no UK tax due — still reportable on SA100 box 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>• Sweden taxes the credited interest at 30% capital rate (Box 7.2 on INK1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>• MISSING rows (Jan-Apr 2025) need earlier statements to complete Swedish 2025 figure.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
UK rental: complete HSBC interest data — Swedish 2025 full £211.26, UK 25/26 full £241.79
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -6024,10 +6024,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="4" min="1" max="1"/>
+    <col width="14" customWidth="1" style="4" min="1" max="1"/>
     <col width="16" customWidth="1" style="4" min="2" max="2"/>
     <col width="22" customWidth="1" style="4" min="3" max="3"/>
     <col width="24" customWidth="1" style="4" min="4" max="4"/>
@@ -6095,100 +6095,128 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>01 Jan 25</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>TO 31DEC2024</t>
         </is>
       </c>
-      <c r="C7" s="19" t="n"/>
-      <c r="D7" s="19" t="n"/>
-      <c r="E7" s="19" t="n"/>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="C7" t="n">
+        <v>4.82</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <f>SUM(C7:D7)</f>
+        <v/>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>24/25</t>
         </is>
       </c>
-      <c r="G7" s="19" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>01 Feb 25</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>TO 31JAN2025</t>
         </is>
       </c>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="19" t="n"/>
-      <c r="F8" s="19" t="inlineStr">
+      <c r="C8" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <f>SUM(C8:D8)</f>
+        <v/>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>24/25</t>
         </is>
       </c>
-      <c r="G8" s="19" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>01 Mar 25</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>TO 28FEB2025</t>
         </is>
       </c>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="19" t="n"/>
-      <c r="F9" s="19" t="inlineStr">
+      <c r="C9" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <f>SUM(C9:D9)</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>24/25</t>
         </is>
       </c>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>01 Apr 25</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>TO 31MAR2025</t>
         </is>
       </c>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="inlineStr">
+      <c r="C10" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="E10">
+        <f>SUM(C10:D10)</f>
+        <v/>
+      </c>
+      <c r="F10" t="inlineStr">
         <is>
           <t>24/25</t>
         </is>
       </c>
-      <c r="G10" s="19" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -6592,7 +6620,6 @@
       <c r="G24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr"/>
       <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Total (£)</t>
@@ -6600,90 +6627,106 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>Coverage</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>UK 25/26 (credits 6 Apr 2025 to 5 Apr 2026)</t>
+          <t>UK 24/25 (partial — Jan-Apr 2025 credits)</t>
         </is>
       </c>
       <c r="B26">
+        <f>SUMIF(F7:F22,"24/25",E7:E22)</f>
+        <v/>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Partial — pre-Jan 2025 not loaded (prior year, not material)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>UK 25/26 (full 12 months)</t>
+        </is>
+      </c>
+      <c r="B27" s="12">
         <f>SUMIF(F7:F22,"25/26",E7:E22)</f>
         <v/>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Full 12 months ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Swedish 2025 (credits Jan-Dec 2025)</t>
-        </is>
-      </c>
-      <c r="B27">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Full year ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Swedish 2025 (full year)</t>
+        </is>
+      </c>
+      <c r="B28" s="12">
         <f>SUMIF(G7:G22,"2025",E7:E22)</f>
         <v/>
       </c>
-      <c r="C27" s="20" t="inlineStr">
-        <is>
-          <t>MISSING Jan-Apr 2025 — partial</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Swedish 2026 partial (Jan-Apr 2026 only)</t>
-        </is>
-      </c>
-      <c r="B28">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Full year ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Swedish 2026 partial (Jan-Apr 2026)</t>
+        </is>
+      </c>
+      <c r="B29">
         <f>SUMIF(G7:G22,"2026",E7:E22)</f>
         <v/>
       </c>
-      <c r="C28" s="16" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>Will need more data later</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="21" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>Notes:</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>• Each month has both a 'GROSS INTEREST TO &lt;date&gt;' line and (sometimes) an 'ADDED GROSS INTEREST' line. Both credit the account.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
         <is>
-          <t>• UK 25/26 PSA covers £1,000 for basic rate; with ~£240 interest, no UK tax due — still reportable on SA100 box 2.</t>
+          <t>• Each month has a GROSS INTEREST line and (sometimes) an ADDED GROSS INTEREST line — both credit the account.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
         <is>
-          <t>• Sweden taxes the credited interest at 30% capital rate (Box 7.2 on INK1).</t>
+          <t>• 01 Apr 25 credit falls in UK 24/25 (before 6 April cutoff); 01 Apr 26 credit falls in UK 25/26.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>• MISSING rows (Jan-Apr 2025) need earlier statements to complete Swedish 2025 figure.</t>
+          <t>• UK 25/26 PSA covers £1,000; with ~£242 interest, no UK tax due — but report on SA100 box 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>• Sweden taxes credited interest at 30% capital rate (Box 7.2 on INK1).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UK rental: full Swedish tax flow (HSBC + CGT) + research findings + filing guide docx
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -76,7 +76,7 @@
       <color rgb="00990000"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -108,6 +108,11 @@
         <fgColor rgb="00FFCCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD966"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -122,7 +127,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,6 +150,8 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5003,13 +5010,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" style="4" min="1" max="1"/>
     <col width="14" customWidth="1" style="4" min="2" max="2"/>
     <col width="15" customWidth="1" style="4" min="3" max="3"/>
-    <col width="30" customWidth="1" style="4" min="4" max="4"/>
+    <col width="35" customWidth="1" style="4" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5560,7 +5567,7 @@
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
         <is>
-          <t>Swedish tax payable on rental property (marginal calc)</t>
+          <t>Swedish 2025 TOTAL capital income tax (all sources)</t>
         </is>
       </c>
       <c r="B59" s="14" t="n"/>
@@ -5571,74 +5578,354 @@
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
         <is>
-          <t>Note: capital income (rental, interest, dividends) is taxed at flat 30% in Sweden.</t>
+          <t>Includes: rental (7.3), HSBC interest (7.2), Vanguard CGT (7.4), mortgage interest (8.1)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
         <is>
-          <t>Other income (salary ~800,000 SEK) is in earned income (~50% marginal); does not affect this calc.</t>
+          <t>All capital income taxed at flat 30% in Sweden. Salary income (~800k SEK) is separate (~50% marginal).</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Net capital income (Box 7.3 - Box 8.1)</t>
-        </is>
-      </c>
-      <c r="B63">
-        <f>$B$44-$B$51</f>
-        <v/>
-      </c>
-      <c r="C63">
-        <f>B63*$B$4</f>
-        <v/>
+      <c r="B63" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="C63" s="12" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="D63" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Capital tax @ 30% (gross, before foreign tax credit)</t>
+          <t>Box 7.2 — Ränteinkomster (HSBC interest, calendar yr)</t>
         </is>
       </c>
       <c r="B64">
-        <f>$B$63*$B$12</f>
+        <f>SUMIF('HSBC Interest'!G:G,"2025",'HSBC Interest'!E:E)</f>
         <v/>
       </c>
       <c r="C64">
         <f>B64*$B$4</f>
         <v/>
       </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>From HSBC Interest tab</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Less: Foreign tax credit</t>
+          <t>Box 7.3 — Överskott vid uthyrning (rental net)</t>
         </is>
       </c>
       <c r="B65">
-        <f>-$B$56</f>
+        <f>$B$44</f>
         <v/>
       </c>
       <c r="C65">
         <f>B65*$B$4</f>
         <v/>
       </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>From rental calc above</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
         <is>
-          <t>Swedish tax payable on this property</t>
-        </is>
-      </c>
-      <c r="B66" s="17">
-        <f>$B$64-$B$56</f>
-        <v/>
-      </c>
-      <c r="C66" s="17">
-        <f>B66*$B$4</f>
+          <t>Box 7.4 — Kapitalvinst (Vanguard ISA sale)</t>
+        </is>
+      </c>
+      <c r="B66" s="12">
+        <f>'Capital Gains 2025'!$B$19</f>
+        <v/>
+      </c>
+      <c r="C66" s="12">
+        <f>'Capital Gains 2025'!$C$19</f>
+        <v/>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>From Capital Gains 2025 tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t>Total capital income</t>
+        </is>
+      </c>
+      <c r="B67" s="15">
+        <f>$B$64+$B$44+$B$66</f>
+        <v/>
+      </c>
+      <c r="C67" s="15">
+        <f>C64+C65+C66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Less: Box 8.1 — Ränteutgifter (mortgage interest)</t>
+        </is>
+      </c>
+      <c r="B68">
+        <f>-$B$51</f>
+        <v/>
+      </c>
+      <c r="C68">
+        <f>-C51</f>
+        <v/>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>From rental calc above</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t>Net capital income (taxable base)</t>
+        </is>
+      </c>
+      <c r="B69" s="12">
+        <f>$B$67-$B$51</f>
+        <v/>
+      </c>
+      <c r="C69" s="12">
+        <f>C67+C68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Swedish capital tax @ 30% (gross, before FTC)</t>
+        </is>
+      </c>
+      <c r="B70">
+        <f>$B$69*$B$12</f>
+        <v/>
+      </c>
+      <c r="C70">
+        <f>C69*$B$12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Less: Foreign tax credit (UK rental tax apportioned)</t>
+        </is>
+      </c>
+      <c r="B71">
+        <f>-$B$56</f>
+        <v/>
+      </c>
+      <c r="C71">
+        <f>-C56</f>
+        <v/>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Only UK property tax — no UK tax on interest (PSA) or CGT (ISA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t>Swedish tax payable for 2025 (rental + interest + CGT)</t>
+        </is>
+      </c>
+      <c r="B72" s="22">
+        <f>C72/$B$4</f>
+        <v/>
+      </c>
+      <c r="C72" s="22">
+        <f>C70+C71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="inlineStr">
+        <is>
+          <t>Note: SEK column is the true tax base. GBP column is informational at year-avg FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr">
+        <is>
+          <t>Memo: tax attributable to each income source (at 30%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rental property (net of interest, after FTC)</t>
+        </is>
+      </c>
+      <c r="B75">
+        <f>($B$44-$B$51)*$B$12-$B$56</f>
+        <v/>
+      </c>
+      <c r="C75">
+        <f>B75*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HSBC interest</t>
+        </is>
+      </c>
+      <c r="B76">
+        <f>$B$64*$B$12</f>
+        <v/>
+      </c>
+      <c r="C76">
+        <f>B76*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Vanguard CGT (no UK tax — ISA)</t>
+        </is>
+      </c>
+      <c r="B77">
+        <f>$B$66*$B$12</f>
+        <v/>
+      </c>
+      <c r="C77">
+        <f>B77*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="23" t="inlineStr">
+        <is>
+          <t>ALTERNATIVE: strict reading uses GROSS rent for schablonavdrag base</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>(Skatteverket guidance says 20% × gross rent, not net of commission)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Gross rent (Swedish 2025)</t>
+        </is>
+      </c>
+      <c r="B81">
+        <f>$B$37</f>
+        <v/>
+      </c>
+      <c r="C81">
+        <f>B81*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Less: 40k SEK std</t>
+        </is>
+      </c>
+      <c r="B82">
+        <f>-$B$10/$B$4</f>
+        <v/>
+      </c>
+      <c r="C82">
+        <f>-$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Less: 20% of GROSS rent</t>
+        </is>
+      </c>
+      <c r="B83">
+        <f>-$B$81*$B$11</f>
+        <v/>
+      </c>
+      <c r="C83">
+        <f>B83*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
+          <t>Box 7.3 — strict gross rent base</t>
+        </is>
+      </c>
+      <c r="B84" s="15">
+        <f>$B$81-$B$10/$B$4-$B$81*$B$11</f>
+        <v/>
+      </c>
+      <c r="C84" s="15">
+        <f>B84*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Difference vs net-of-commission method</t>
+        </is>
+      </c>
+      <c r="B85">
+        <f>$B$84-$B$44</f>
+        <v/>
+      </c>
+      <c r="C85">
+        <f>B85*$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Extra Swedish tax if strict method applied (30%)</t>
+        </is>
+      </c>
+      <c r="B86" s="19">
+        <f>($B$84-$B$44)*$B$12</f>
+        <v/>
+      </c>
+      <c r="C86" s="19">
+        <f>B86*$B$4</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
UK rental: rebuild CGT with genomsnittsmetoden using actual Vanguard contribution history
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -10,8 +10,8 @@
     <sheet name="Santander" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Tax 24-25" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Tax 25-26" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Capital Gains 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="HSBC Interest" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="HSBC Interest" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Capital Gains 2025" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -76,7 +76,7 @@
       <color rgb="00990000"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +113,11 @@
         <fgColor rgb="00FFD966"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -127,7 +132,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,6 +157,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5653,11 +5659,11 @@
         </is>
       </c>
       <c r="B66" s="12">
-        <f>'Capital Gains 2025'!$B$19</f>
+        <f>'Capital Gains 2025'!$B$33</f>
         <v/>
       </c>
       <c r="C66" s="12">
-        <f>'Capital Gains 2025'!$C$19</f>
+        <f>'Capital Gains 2025'!$C$33</f>
         <v/>
       </c>
       <c r="D66" t="inlineStr">
@@ -5938,374 +5944,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E43"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="60" customWidth="1" style="4" min="1" max="1"/>
-    <col width="16" customWidth="1" style="4" min="2" max="2"/>
-    <col width="16" customWidth="1" style="4" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Capital Gains 2025 — Vanguard ISA (sold June 2025)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>Held in UK ISA → no UK tax. Swedish residency 25 Nov 2021 → cost basis taken at that date.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>Swedish capital gains tax: 30% flat on net gain in SEK.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Parameters (edit to recalc):</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="n"/>
-      <c r="C6" s="14" t="n"/>
-      <c r="D6" s="14" t="n"/>
-      <c r="E6" s="14" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Cost basis date</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>25 Nov 2021</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>(Swedish tax-residency start)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Cost basis value (GBP)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>23031.31</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Cost basis FX rate (Nov 2021)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>11.84728</v>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>Riksbanken Nov 2021 monthly avg</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Sale date</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>5 Jun 2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Sale proceeds (GBP)</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>29862.97</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Sale FX rate (Jun 2025)</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>12.9485</v>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>Riksbanken Jun 2025 monthly avg</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Swedish capital tax rate</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Calculation</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
-      <c r="E15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>SEK</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Cost basis (omkostnadsbelopp)</t>
-        </is>
-      </c>
-      <c r="B17">
-        <f>$B$8</f>
-        <v/>
-      </c>
-      <c r="C17">
-        <f>$B$8*$B$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Sale proceeds (försäljningspris)</t>
-        </is>
-      </c>
-      <c r="B18">
-        <f>$B$11</f>
-        <v/>
-      </c>
-      <c r="C18">
-        <f>$B$11*$B$12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Capital gain</t>
-        </is>
-      </c>
-      <c r="B19" s="15">
-        <f>$B$11-$B$8</f>
-        <v/>
-      </c>
-      <c r="C19" s="15">
-        <f>$B$11*$B$12-$B$8*$B$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>Decomposition (memo):</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Investment performance in GBP</t>
-        </is>
-      </c>
-      <c r="B22">
-        <f>$B$11-$B$8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FX uplift on cost basis (Nov21 → Jun25)</t>
-        </is>
-      </c>
-      <c r="C23">
-        <f>$B$8*($B$12-$B$9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  → Total SEK gain (matches above)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Swedish capital tax (30% of SEK gain)</t>
-        </is>
-      </c>
-      <c r="B26" s="17">
-        <f>$C$19*$B$13/$B$12</f>
-        <v/>
-      </c>
-      <c r="C26" s="17">
-        <f>$C$19*$B$13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>Reporting in your Swedish tax return:</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>• File K4 (bilaga K4) — avsnitt A or C depending on whether marknadsnoterade aktier/fonder</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>• K4 lists: antal/units, försäljningspris, omkostnadsbelopp, vinst</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>• Net gain rolls into Box 7.4 (kapitalvinst marknadsnoterade aktier/fonder) on INK1</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>• Box 7.2 catches general interest/dividends; CGT-specific lines are 7.4/7.5/7.6 depending on type</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="13" t="inlineStr">
-        <is>
-          <t>Assumptions &amp; caveats:</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="n"/>
-      <c r="C35" s="14" t="n"/>
-      <c r="D35" s="14" t="n"/>
-      <c r="E35" s="14" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="16" t="inlineStr">
-        <is>
-          <t>• Cost basis taken at 25 Nov 2021 value (Swedish residency start). This is the simplest approach if</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  the bulk of the holding pre-dated the move. If significant contributions were made AFTER Nov 2021,</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Swedish tax law applies the average-cost method (genomsnittsmetoden) — each contribution's own</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  cost basis (in SEK at the time) is weighted into the average. Confirm with accountant if you</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  contributed materially between Nov 2021 and Jun 2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t>• FX rates used are Riksbanken monthly averages for Nov 2021 and Jun 2025.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t>• ISA wrapper provides no Swedish tax benefit — Sweden taxes the gain regardless.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t>• Capital losses elsewhere in the same year can offset this gain (currently none assumed).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7023,4 +6661,630 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" style="4" min="1" max="1"/>
+    <col width="18" customWidth="1" style="4" min="2" max="2"/>
+    <col width="20" customWidth="1" style="4" min="3" max="3"/>
+    <col width="38" customWidth="1" style="4" min="4" max="4"/>
+    <col width="18" customWidth="1" style="4" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Vanguard ISA — Capital Gains 2025 (genomsnittsmetoden)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Per Swedish tax law: cost basis = original acquisition cost in SEK at original-date FX rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>No rebasing on Swedish residency move. All contributions were Sep 2020 to Oct 2021 (no contributions after Nov 2021 move).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>FX rates in yellow cells — approximate; verify against Riksbanken monthly averages and overwrite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Contribution (£)</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Monthly avg FX (SEK/GBP)</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>SEK cost basis</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sep 2020</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>200</v>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E8">
+        <f>B8*C8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Oct 2020</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2508.82</v>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E9">
+        <f>B9*C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nov 2020</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>200</v>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E10">
+        <f>B10*C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dec 2020</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>200</v>
+      </c>
+      <c r="C11" s="24" t="n">
+        <v>11.21</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E11">
+        <f>B11*C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Jan 2021</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>200</v>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E12">
+        <f>B12*C12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>9800</v>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E13">
+        <f>B13*C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>800</v>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E14">
+        <f>B14*C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Apr 2021</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>800</v>
+      </c>
+      <c r="C15" s="24" t="n">
+        <v>11.74</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E15">
+        <f>B15*C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>May 2021</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>800</v>
+      </c>
+      <c r="C16" s="24" t="n">
+        <v>11.78</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E16">
+        <f>B16*C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Jun 2021</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>800</v>
+      </c>
+      <c r="C17" s="24" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E17">
+        <f>B17*C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Jul 2021</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>800</v>
+      </c>
+      <c r="C18" s="24" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E18">
+        <f>B18*C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Aug 2021</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>800</v>
+      </c>
+      <c r="C19" s="24" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E19">
+        <f>B19*C19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sep 2021</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>800</v>
+      </c>
+      <c r="C20" s="24" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E20">
+        <f>B20*C20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Oct 2021</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>800</v>
+      </c>
+      <c r="C21" s="24" t="n">
+        <v>11.89</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Riksbanken monthly avg (estimate, verify)</t>
+        </is>
+      </c>
+      <c r="E21">
+        <f>B21*C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>Total contributions</t>
+        </is>
+      </c>
+      <c r="B22" s="15">
+        <f>SUM(B8:B21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="15">
+        <f>SUM(E8:E21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>Sale 5 June 2025</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="14" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sale proceeds (£)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>29862.97</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>June 2025 monthly avg FX (SEK/GBP)</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="n">
+        <v>12.9485</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Riksbanken Jun 2025 monthly avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Sale proceeds (SEK)</t>
+        </is>
+      </c>
+      <c r="B27" s="15">
+        <f>$B$25*$B$26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Sale proceeds</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>$B$25</f>
+        <v/>
+      </c>
+      <c r="C31">
+        <f>$B$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Less: Omkostnadsbelopp (sum of contributions in SEK)</t>
+        </is>
+      </c>
+      <c r="B32">
+        <f>-$B$22</f>
+        <v/>
+      </c>
+      <c r="C32">
+        <f>-$E$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Capital gain</t>
+        </is>
+      </c>
+      <c r="B33" s="15">
+        <f>$B$25-$B$22</f>
+        <v/>
+      </c>
+      <c r="C33" s="15">
+        <f>$B$27-$E$22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Swedish capital tax (30%)</t>
+        </is>
+      </c>
+      <c r="B35" s="17">
+        <f>$C$33*0.30/$B$26</f>
+        <v/>
+      </c>
+      <c r="C35" s="17">
+        <f>$C$33*0.30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>Genomsnittsmetoden (weighted-average) cost basis</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="n"/>
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="14" t="n"/>
+      <c r="E38" s="14" t="n"/>
+      <c r="F38" s="14" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>• Sweden uses genomsnittsmetoden: each contribution's cost basis is the GBP × FX at acquisition date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>• Since the user sold ALL units in June 2025, the cost basis is simply the SEK sum of all contributions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>• No rebasing on becoming Swedish resident (Nov 2021).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>• Reference: 44 kap. 14 § Inkomstskattelagen; Skatteverket 'Utländsk valuta' guidance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>• Yellow FX cells are estimates — verify against riksbank.se/sv/statistik/rantor-och-valutakurser/sok-rantor-och-valutakurser/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>Reporting on Swedish tax return (INK1)</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="14" t="n"/>
+      <c r="E45" s="14" t="n"/>
+      <c r="F45" s="14" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>• File K4 avsnitt A — list units sold, försäljningspris (sale SEK), omkostnadsbelopp (cost SEK), vinst</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>• Net gain rolls into Box 7.4 (kapitalvinst marknadsnoterade aktier/fonder)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr">
+        <is>
+          <t>• ISA wrapper is irrelevant for Swedish tax — full gain taxable</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr">
+        <is>
+          <t>• Capital losses elsewhere in 2025 can offset (100% against listed shares, 70% against other capital)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
UK rental: refine tax positions — leasehold=privatbostadsfastighet, net-of-commission defensible, fee not deductible
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -6686,7 +6686,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -6708,7 +6707,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
         <is>
@@ -7060,7 +7058,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="13" t="inlineStr">
         <is>
@@ -7109,7 +7106,6 @@
         <v/>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
UK rental: add Yield Analysis tab — gross/NOI/cash-on-cash/total return
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Tax 25-26" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="HSBC Interest" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Capital Gains 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Yield Analysis" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -132,7 +133,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,6 +159,10 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7283,4 +7288,562 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" style="4" min="1" max="1"/>
+    <col width="14" customWidth="1" style="4" min="2" max="2"/>
+    <col width="17" customWidth="1" style="4" min="3" max="3"/>
+    <col width="15" customWidth="1" style="4" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>76a Ingelow Road — Investment Yield Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Assuming gross-of-commission position for Swedish tax (£1,215 more conservative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Inputs (edit to update yields)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="14" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Property purchase price (2018)</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>635000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Years held (to 2025)</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Current property value</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Current mortgage outstanding (interest only)</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>178764.94</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Equity in property (= value − mortgage)</t>
+        </is>
+      </c>
+      <c r="B9" s="15">
+        <f>$B$7-$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Eventual CGT assumption (on current £165k appreciation)</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Historical CAGR (from 2018 purchase)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Total appreciation (current − purchase)</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>$B$7-$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Effective CGT rate on appreciation</t>
+        </is>
+      </c>
+      <c r="B14" s="25">
+        <f>$B$10/($B$7-$B$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>CAGR (annualised)</t>
+        </is>
+      </c>
+      <c r="B15" s="26">
+        <f>($B$7/$B$5)^(1/$B$6)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Forward annual appreciation (at CAGR × current value)</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>$B$7*$B$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Forward appreciation AFTER CGT</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>$B$16*(1-$B$14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Income statement 2025 (gross-of-commission Swedish, product fee in 2025)</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="14" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Gross rental income (UK 25/26)</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>'Tax 25-26'!$B$16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Knight Frank commission</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>'Tax 25-26'!$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Repairs &amp; maintenance</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>'Tax 25-26'!$B$19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mortgage interest</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>-'Tax 25-26'!$B$23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Mortgage product fee (one-off, 2025)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>-'Tax 25-26'!$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>UK tax on rental (net of finance credit)</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>-'Tax 25-26'!$B$32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Swedish tax on rental (gross-of-commission base, less FTC)</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>-((0.80*'Tax 25-26'!$B$37-'Tax 25-26'!$B$10/'Tax 25-26'!$B$4-'Tax 25-26'!$B$51)*0.30-'Tax 25-26'!$B$56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Net cash income after all costs and tax (2025)</t>
+        </is>
+      </c>
+      <c r="B28" s="17">
+        <f>$B$21+$B$22+$B$23+$B$24+$B$25+$B$26+$B$27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Yield metrics</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>% on current value</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>% on equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Gross yield (rent / value)</t>
+        </is>
+      </c>
+      <c r="B32">
+        <f>$B$21</f>
+        <v/>
+      </c>
+      <c r="C32" s="25">
+        <f>B32/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Net Operating Income (NOI — pre-leverage, pre-tax)</t>
+        </is>
+      </c>
+      <c r="B33">
+        <f>$B$21+$B$22+$B$23</f>
+        <v/>
+      </c>
+      <c r="C33" s="25">
+        <f>B33/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Net cash income (post all costs + tax, 2025)</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>$B$28</f>
+        <v/>
+      </c>
+      <c r="C34" s="25">
+        <f>B34/$B$7</f>
+        <v/>
+      </c>
+      <c r="D34" s="25">
+        <f>B34/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Steady-state cash income (excl. product fee)</t>
+        </is>
+      </c>
+      <c r="B36">
+        <f>$B$28-$B$25</f>
+        <v/>
+      </c>
+      <c r="C36" s="25">
+        <f>B36/$B$7</f>
+        <v/>
+      </c>
+      <c r="D36" s="25">
+        <f>B36/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Forward annual appreciation (CAGR × current value)</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>$B$16</f>
+        <v/>
+      </c>
+      <c r="C38" s="25">
+        <f>B38/$B$7</f>
+        <v/>
+      </c>
+      <c r="D38" s="25">
+        <f>B38/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Total return — pre-CGT (steady cash + forward appreciation)</t>
+        </is>
+      </c>
+      <c r="B39" s="17">
+        <f>$B$36+$B$16</f>
+        <v/>
+      </c>
+      <c r="C39" s="27">
+        <f>B39/$B$7</f>
+        <v/>
+      </c>
+      <c r="D39" s="28">
+        <f>B39/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Total return — POST-CGT (steady cash + post-CGT appreciation)</t>
+        </is>
+      </c>
+      <c r="B40" s="17">
+        <f>$B$36+$B$17</f>
+        <v/>
+      </c>
+      <c r="C40" s="27">
+        <f>B40/$B$7</f>
+        <v/>
+      </c>
+      <c r="D40" s="28">
+        <f>B40/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>Benchmarks (rough reference)</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14" t="n"/>
+      <c r="E42" s="14" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>UK 10-year gilts (risk-free)</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>~4-5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>UK cash savings (instant access)</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>~4-5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>UK FTSE 100 long-term nominal</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>~7-8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>Global equity index (long-term)</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>~7-9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>Your Vanguard ISA return (2020-2025)</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>~10%/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="n"/>
+      <c r="C49" s="14" t="n"/>
+      <c r="D49" s="14" t="n"/>
+      <c r="E49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>• 'Cash-on-cash' divides by equity, reflecting that you've only got ~£621k of own money in the flat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>• 'NOI yield' is pre-leverage — useful for comparing flats to other property investments before mortgage effects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t>• Total return reflects assumption that 2018-2025 CAGR continues forward. London may not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>• Post-CGT applies the implied 14.5% effective CGT rate (£24k on £165k gain) to forward appreciation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>• Excludes: voids, refurbishment beyond annual maintenance, mortgage refinance risk after May 2027 (rate may rise from 4.38%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>• Excludes: opportunity cost of equity. If £621k earned 5% in gilts = £31k/year passive — almost matches the steady-state cash yield.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
UK rental: add 0% appreciation scenario to Yield tab
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -7296,7 +7296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" style="4" min="1" max="1"/>
@@ -7319,6 +7319,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -7391,6 +7392,7 @@
         <v>24000</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
@@ -7457,6 +7459,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
@@ -7563,6 +7566,7 @@
         <v/>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
@@ -7640,6 +7644,7 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
@@ -7838,6 +7843,79 @@
         <is>
           <t>• Excludes: opportunity cost of equity. If £621k earned 5% in gilts = £31k/year passive — almost matches the steady-state cash yield.</t>
         </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>Zero-appreciation scenario (assume £0 capital growth)</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="14" t="n"/>
+      <c r="E58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>(Conservative — reflects flat-to-down London market recent years)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>% on value</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>% on equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Total return — 2025 cash only (with fee, 0% appreciation)</t>
+        </is>
+      </c>
+      <c r="B62">
+        <f>$B$34</f>
+        <v/>
+      </c>
+      <c r="C62" s="25">
+        <f>B62/$B$7</f>
+        <v/>
+      </c>
+      <c r="D62" s="25">
+        <f>B62/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>Total return — steady-state cash only (excl fee, 0% appreciation)</t>
+        </is>
+      </c>
+      <c r="B63" s="17">
+        <f>$B$36</f>
+        <v/>
+      </c>
+      <c r="C63" s="28">
+        <f>B63/$B$7</f>
+        <v/>
+      </c>
+      <c r="D63" s="28">
+        <f>B63/$B$9</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UK rental: lock in conservative positions (gross rent, no fee, genomsnittsmetoden) in both xlsx and docx
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -5021,7 +5021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E86"/>
+  <dimension ref="A1:E90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" style="4" min="1" max="1"/>
@@ -5386,16 +5386,16 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>Rental income net of commission (basis for schablonavdrag)</t>
-        </is>
-      </c>
-      <c r="B39" s="15">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>(Memo: rental income net of commission — NOT used; gross applies)</t>
+        </is>
+      </c>
+      <c r="B39" s="12">
         <f>$B$37+$B$38</f>
         <v/>
       </c>
-      <c r="C39" s="15">
+      <c r="C39" s="12">
         <f>B39*$B$4</f>
         <v/>
       </c>
@@ -5403,7 +5403,7 @@
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
-          <t>Schablonavdrag (replaces actual expense deduction):</t>
+          <t>Schablonavdrag (applied to GROSS rent per Skatteverket strict reading):</t>
         </is>
       </c>
     </row>
@@ -5425,11 +5425,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  20% of rental income (net of commission)</t>
+          <t xml:space="preserve">  20% of GROSS rent</t>
         </is>
       </c>
       <c r="B43">
-        <f>-$B$39*$B$11</f>
+        <f>-$B$37*$B$11</f>
         <v/>
       </c>
       <c r="C43">
@@ -5444,7 +5444,7 @@
         </is>
       </c>
       <c r="B44" s="17">
-        <f>$B$39+$B$42+$B$43</f>
+        <f>$B$37+$B$42+$B$43</f>
         <v/>
       </c>
       <c r="C44" s="17">
@@ -5490,28 +5490,26 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Mortgage product fees (deductible)</t>
-        </is>
-      </c>
-      <c r="B50">
-        <f>SUMIF('Santander'!$B$4:$AN$4,$C$6,'Santander'!$B$8:$AN$8)</f>
-        <v/>
-      </c>
-      <c r="C50">
-        <f>B50*$B$4</f>
-        <v/>
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>Mortgage product fees (NOT deductible per RÅ 1997 ref. 63)</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
         <is>
-          <t>Box 8.1 total</t>
+          <t>Box 8.1 total (interest only — product fee excluded)</t>
         </is>
       </c>
       <c r="B51" s="17">
-        <f>$B$49+$B$50</f>
+        <f>$B$49</f>
         <v/>
       </c>
       <c r="C51" s="17">
@@ -5836,110 +5834,92 @@
         <v/>
       </c>
     </row>
+    <row r="78"/>
     <row r="79">
       <c r="A79" s="23" t="inlineStr">
         <is>
-          <t>ALTERNATIVE: strict reading uses GROSS rent for schablonavdrag base</t>
+          <t>ALTERNATIVE: filed-position scenario using net-of-commission base</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
         <is>
-          <t>(Skatteverket guidance says 20% × gross rent, not net of commission)</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Gross rent (Swedish 2025)</t>
-        </is>
-      </c>
-      <c r="B81">
-        <f>$B$37</f>
-        <v/>
-      </c>
-      <c r="C81">
-        <f>B81*$B$4</f>
-        <v/>
-      </c>
-    </row>
+          <t>(Less conservative — matches 2024 filing approach. Differential vs current strict position shown below.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81"/>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Less: 40k SEK std</t>
+          <t>Net rental (after commission)</t>
         </is>
       </c>
       <c r="B82">
-        <f>-$B$10/$B$4</f>
-        <v/>
-      </c>
-      <c r="C82">
-        <f>-$B$10</f>
+        <f>$B$37+$B$38</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Less: 20% of GROSS rent</t>
+          <t>Less: 40k SEK std</t>
         </is>
       </c>
       <c r="B83">
-        <f>-$B$81*$B$11</f>
-        <v/>
-      </c>
-      <c r="C83">
-        <f>B83*$B$4</f>
+        <f>-$B$10/$B$4</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t>Box 7.3 — strict gross rent base</t>
-        </is>
-      </c>
-      <c r="B84" s="15">
-        <f>$B$81-$B$10/$B$4-$B$81*$B$11</f>
-        <v/>
-      </c>
-      <c r="C84" s="15">
-        <f>B84*$B$4</f>
-        <v/>
-      </c>
+          <t>Less: 20% of NET rental</t>
+        </is>
+      </c>
+      <c r="B84" s="12">
+        <f>-($B$37+$B$38)*$B$11</f>
+        <v/>
+      </c>
+      <c r="C84" s="12" t="n"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Difference vs net-of-commission method</t>
+          <t>Plus: Product fee deduction in Box 8.1 (alternative)</t>
         </is>
       </c>
       <c r="B85">
-        <f>$B$84-$B$44</f>
-        <v/>
-      </c>
-      <c r="C85">
-        <f>B85*$B$4</f>
+        <f>-SUMIF('Santander'!$B$4:$AN$4,$C$6,'Santander'!$B$8:$AN$8)</f>
         <v/>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Extra Swedish tax if strict method applied (30%)</t>
-        </is>
-      </c>
-      <c r="B86" s="19">
-        <f>($B$84-$B$44)*$B$12</f>
-        <v/>
-      </c>
-      <c r="C86" s="19">
-        <f>B86*$B$4</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A86" s="12" t="inlineStr">
+        <is>
+          <t>Alternative Box 7.3 (net-of-commission)</t>
+        </is>
+      </c>
+      <c r="B86" s="12">
+        <f>($B$37+$B$38)+(-$B$10/$B$4)+(-($B$37+$B$38)*$B$11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Tax saving if alternative applied (30% of differential)</t>
+        </is>
+      </c>
+      <c r="B87" s="19">
+        <f>($B$44-$B$86+SUMIF('Santander'!$B$4:$AN$4,$C$6,'Santander'!$B$8:$AN$8))*0.30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
@@ -7319,7 +7299,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -7392,7 +7371,6 @@
         <v>24000</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
@@ -7459,7 +7437,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
@@ -7566,7 +7543,6 @@
         <v/>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="13" t="inlineStr">
         <is>
@@ -7644,7 +7620,6 @@
         <v/>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Rebuild Tax_Return.xlsx Capital Gains 2025 tab — per-fund genomsnittsmetoden, formatted, total SEK 150,150
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Tax 24-25" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Tax 25-26" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="HSBC Interest" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Capital Gains 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Yield Analysis" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Yield Analysis" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Capital Gains 2025" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -21,11 +21,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -76,8 +78,21 @@
     <font>
       <color rgb="00990000"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -119,6 +134,26 @@
         <fgColor rgb="00FFFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005B9BD5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -133,7 +168,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -163,6 +198,31 @@
     <xf numFmtId="10" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="11" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="11" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="11" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="12" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="12" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="12" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="12" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5021,7 +5081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" style="4" min="1" max="1"/>
@@ -5037,6 +5097,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -5153,6 +5214,7 @@
         <v>0.3</v>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
@@ -5226,6 +5288,7 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
@@ -5266,6 +5329,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
@@ -5332,6 +5396,8 @@
         <v/>
       </c>
     </row>
+    <row r="33"/>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
@@ -5400,6 +5466,7 @@
         <v/>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
@@ -5452,6 +5519,7 @@
         <v/>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
@@ -5463,6 +5531,7 @@
         <v/>
       </c>
     </row>
+    <row r="47"/>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
@@ -5517,6 +5586,7 @@
         <v/>
       </c>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
         <is>
@@ -5573,6 +5643,8 @@
         <v/>
       </c>
     </row>
+    <row r="57"/>
+    <row r="58"/>
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
         <is>
@@ -5598,6 +5670,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63">
       <c r="B63" s="12" t="inlineStr">
         <is>
@@ -5662,11 +5735,11 @@
         </is>
       </c>
       <c r="B66" s="12">
-        <f>'Capital Gains 2025'!$B$33</f>
+        <f>'Capital Gains 2025'!$C$17</f>
         <v/>
       </c>
       <c r="C66" s="12">
-        <f>'Capital Gains 2025'!$C$33</f>
+        <f>'Capital Gains 2025'!$C$17</f>
         <v/>
       </c>
       <c r="D66" t="inlineStr">
@@ -5834,7 +5907,6 @@
         <v/>
       </c>
     </row>
-    <row r="78"/>
     <row r="79">
       <c r="A79" s="23" t="inlineStr">
         <is>
@@ -5849,7 +5921,6 @@
         </is>
       </c>
     </row>
-    <row r="81"/>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
@@ -5917,9 +5988,6 @@
         <v/>
       </c>
     </row>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>
@@ -6654,617 +6722,626 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" style="4" min="1" max="1"/>
-    <col width="18" customWidth="1" style="4" min="2" max="2"/>
-    <col width="20" customWidth="1" style="4" min="3" max="3"/>
-    <col width="38" customWidth="1" style="4" min="4" max="4"/>
-    <col width="18" customWidth="1" style="4" min="5" max="5"/>
+    <col width="62" customWidth="1" style="4" min="1" max="1"/>
+    <col width="14" customWidth="1" style="4" min="2" max="2"/>
+    <col width="17" customWidth="1" style="4" min="3" max="3"/>
+    <col width="15" customWidth="1" style="4" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Vanguard ISA — Capital Gains 2025 (genomsnittsmetoden)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>Per Swedish tax law: cost basis = original acquisition cost in SEK at original-date FX rate.</t>
+          <t>76a Ingelow Road — Investment Yield Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Assuming gross-of-commission position for Swedish tax (£1,215 more conservative)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>No rebasing on Swedish residency move. All contributions were Sep 2020 to Oct 2021 (no contributions after Nov 2021 move).</t>
-        </is>
-      </c>
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Inputs (edit to update yields)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="14" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>FX rates in yellow cells — approximate; verify against Riksbanken monthly averages and overwrite.</t>
-        </is>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Property purchase price (2018)</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>635000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Years held (to 2025)</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Contribution (£)</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>Monthly avg FX (SEK/GBP)</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>SEK cost basis</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Current property value</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="n">
+        <v>800000</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Sep 2020</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>200</v>
-      </c>
-      <c r="C8" s="24" t="n">
-        <v>11.34</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E8">
-        <f>B8*C8</f>
-        <v/>
+          <t>Current mortgage outstanding (interest only)</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>178764.94</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Oct 2020</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>2508.82</v>
-      </c>
-      <c r="C9" s="24" t="n">
-        <v>11.27</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E9">
-        <f>B9*C9</f>
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Equity in property (= value − mortgage)</t>
+        </is>
+      </c>
+      <c r="B9" s="15">
+        <f>$B$7-$B$8</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nov 2020</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>200</v>
-      </c>
-      <c r="C10" s="24" t="n">
-        <v>11.34</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E10">
-        <f>B10*C10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Dec 2020</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>200</v>
-      </c>
-      <c r="C11" s="24" t="n">
-        <v>11.21</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E11">
-        <f>B11*C11</f>
-        <v/>
+          <t>Eventual CGT assumption (on current £165k appreciation)</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>24000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Jan 2021</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>200</v>
-      </c>
-      <c r="C12" s="24" t="n">
-        <v>11.34</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E12">
-        <f>B12*C12</f>
-        <v/>
-      </c>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Historical CAGR (from 2018 purchase)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Feb 2021</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>9800</v>
-      </c>
-      <c r="C13" s="24" t="n">
-        <v>11.78</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E13">
-        <f>B13*C13</f>
+          <t>Total appreciation (current − purchase)</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>$B$7-$B$5</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mar 2021</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>800</v>
-      </c>
-      <c r="C14" s="24" t="n">
-        <v>11.78</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E14">
-        <f>B14*C14</f>
+          <t>Effective CGT rate on appreciation</t>
+        </is>
+      </c>
+      <c r="B14" s="25">
+        <f>$B$10/($B$7-$B$5)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Apr 2021</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>800</v>
-      </c>
-      <c r="C15" s="24" t="n">
-        <v>11.74</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E15">
-        <f>B15*C15</f>
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>CAGR (annualised)</t>
+        </is>
+      </c>
+      <c r="B15" s="26">
+        <f>($B$7/$B$5)^(1/$B$6)-1</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>May 2021</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>800</v>
-      </c>
-      <c r="C16" s="24" t="n">
-        <v>11.78</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E16">
-        <f>B16*C16</f>
+          <t>Forward annual appreciation (at CAGR × current value)</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>$B$7*$B$15</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Jun 2021</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>800</v>
-      </c>
-      <c r="C17" s="24" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E17">
-        <f>B17*C17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Jul 2021</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>800</v>
-      </c>
-      <c r="C18" s="24" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E18">
-        <f>B18*C18</f>
+          <t>Forward appreciation AFTER CGT</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>$B$16*(1-$B$14)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Aug 2021</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>800</v>
-      </c>
-      <c r="C19" s="24" t="n">
-        <v>11.95</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E19">
-        <f>B19*C19</f>
-        <v/>
-      </c>
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Income statement 2025 (gross-of-commission Swedish, product fee in 2025)</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="14" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Sep 2021</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>800</v>
-      </c>
-      <c r="C20" s="24" t="n">
-        <v>11.92</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E20">
-        <f>B20*C20</f>
-        <v/>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Oct 2021</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>800</v>
-      </c>
-      <c r="C21" s="24" t="n">
-        <v>11.89</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Riksbanken monthly avg (estimate, verify)</t>
-        </is>
-      </c>
-      <c r="E21">
-        <f>B21*C21</f>
+          <t>Gross rental income (UK 25/26)</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>'Tax 25-26'!$B$16</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>Total contributions</t>
-        </is>
-      </c>
-      <c r="B22" s="15">
-        <f>SUM(B8:B21)</f>
-        <v/>
-      </c>
-      <c r="E22" s="15">
-        <f>SUM(E8:E21)</f>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Knight Frank commission</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>'Tax 25-26'!$B$17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Repairs &amp; maintenance</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>'Tax 25-26'!$B$19</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>Sale 5 June 2025</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mortgage interest</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>-'Tax 25-26'!$B$23</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sale proceeds (£)</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>29862.97</v>
+          <t>Mortgage product fee (one-off, 2025)</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>-'Tax 25-26'!$B$24</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>June 2025 monthly avg FX (SEK/GBP)</t>
-        </is>
-      </c>
-      <c r="B26" s="24" t="n">
-        <v>12.9485</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Riksbanken Jun 2025 monthly avg</t>
-        </is>
+          <t>UK tax on rental (net of finance credit)</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>-'Tax 25-26'!$B$32</f>
+        <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>Sale proceeds (SEK)</t>
-        </is>
-      </c>
-      <c r="B27" s="15">
-        <f>$B$25*$B$26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
-        <is>
-          <t>Calculation</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="14" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Swedish tax on rental (gross-of-commission base, less FTC)</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>-((0.80*'Tax 25-26'!$B$37-'Tax 25-26'!$B$10/'Tax 25-26'!$B$4-'Tax 25-26'!$B$51)*0.30-'Tax 25-26'!$B$56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Net cash income after all costs and tax (2025)</t>
+        </is>
+      </c>
+      <c r="B28" s="17">
+        <f>$B$21+$B$22+$B$23+$B$24+$B$25+$B$26+$B$27</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="inlineStr">
-        <is>
-          <t>SEK</t>
-        </is>
-      </c>
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>Yield metrics</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Sale proceeds</t>
-        </is>
-      </c>
-      <c r="B31">
-        <f>$B$25</f>
-        <v/>
-      </c>
-      <c r="C31">
-        <f>$B$27</f>
-        <v/>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>% on current value</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>% on equity</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Less: Omkostnadsbelopp (sum of contributions in SEK)</t>
+          <t>Gross yield (rent / value)</t>
         </is>
       </c>
       <c r="B32">
-        <f>-$B$22</f>
-        <v/>
-      </c>
-      <c r="C32">
-        <f>-$E$22</f>
+        <f>$B$21</f>
+        <v/>
+      </c>
+      <c r="C32" s="25">
+        <f>B32/$B$7</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t>Capital gain</t>
-        </is>
-      </c>
-      <c r="B33" s="15">
-        <f>$B$25-$B$22</f>
-        <v/>
-      </c>
-      <c r="C33" s="15">
-        <f>$B$27-$E$22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>Swedish capital tax (30%)</t>
-        </is>
-      </c>
-      <c r="B35" s="17">
-        <f>$C$33*0.30/$B$26</f>
-        <v/>
-      </c>
-      <c r="C35" s="17">
-        <f>$C$33*0.30</f>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Net Operating Income (NOI — pre-leverage, pre-tax)</t>
+        </is>
+      </c>
+      <c r="B33">
+        <f>$B$21+$B$22+$B$23</f>
+        <v/>
+      </c>
+      <c r="C33" s="25">
+        <f>B33/$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Net cash income (post all costs + tax, 2025)</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>$B$28</f>
+        <v/>
+      </c>
+      <c r="C34" s="25">
+        <f>B34/$B$7</f>
+        <v/>
+      </c>
+      <c r="D34" s="25">
+        <f>B34/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Steady-state cash income (excl. product fee)</t>
+        </is>
+      </c>
+      <c r="B36">
+        <f>$B$28-$B$25</f>
+        <v/>
+      </c>
+      <c r="C36" s="25">
+        <f>B36/$B$7</f>
+        <v/>
+      </c>
+      <c r="D36" s="25">
+        <f>B36/$B$9</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>Genomsnittsmetoden (weighted-average) cost basis</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="14" t="n"/>
-      <c r="D38" s="14" t="n"/>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="14" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Forward annual appreciation (CAGR × current value)</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>$B$16</f>
+        <v/>
+      </c>
+      <c r="C38" s="25">
+        <f>B38/$B$7</f>
+        <v/>
+      </c>
+      <c r="D38" s="25">
+        <f>B38/$B$9</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="inlineStr">
-        <is>
-          <t>• Sweden uses genomsnittsmetoden: each contribution's cost basis is the GBP × FX at acquisition date.</t>
-        </is>
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>Total return — pre-CGT (steady cash + forward appreciation)</t>
+        </is>
+      </c>
+      <c r="B39" s="17">
+        <f>$B$36+$B$16</f>
+        <v/>
+      </c>
+      <c r="C39" s="27">
+        <f>B39/$B$7</f>
+        <v/>
+      </c>
+      <c r="D39" s="28">
+        <f>B39/$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="inlineStr">
-        <is>
-          <t>• Since the user sold ALL units in June 2025, the cost basis is simply the SEK sum of all contributions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="16" t="inlineStr">
-        <is>
-          <t>• No rebasing on becoming Swedish resident (Nov 2021).</t>
-        </is>
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Total return — POST-CGT (steady cash + post-CGT appreciation)</t>
+        </is>
+      </c>
+      <c r="B40" s="17">
+        <f>$B$36+$B$17</f>
+        <v/>
+      </c>
+      <c r="C40" s="27">
+        <f>B40/$B$7</f>
+        <v/>
+      </c>
+      <c r="D40" s="28">
+        <f>B40/$B$9</f>
+        <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t>• Reference: 44 kap. 14 § Inkomstskattelagen; Skatteverket 'Utländsk valuta' guidance.</t>
-        </is>
-      </c>
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>Benchmarks (rough reference)</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14" t="n"/>
+      <c r="E42" s="14" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
         <is>
-          <t>• Yellow FX cells are estimates — verify against riksbank.se/sv/statistik/rantor-och-valutakurser/sok-rantor-och-valutakurser/</t>
+          <t>UK 10-year gilts (risk-free)</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>~4-5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>UK cash savings (instant access)</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>~4-5%</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="inlineStr">
-        <is>
-          <t>Reporting on Swedish tax return (INK1)</t>
-        </is>
-      </c>
-      <c r="B45" s="14" t="n"/>
-      <c r="C45" s="14" t="n"/>
-      <c r="D45" s="14" t="n"/>
-      <c r="E45" s="14" t="n"/>
-      <c r="F45" s="14" t="n"/>
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>UK FTSE 100 long-term nominal</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>~7-8%</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
-          <t>• File K4 avsnitt A — list units sold, försäljningspris (sale SEK), omkostnadsbelopp (cost SEK), vinst</t>
+          <t>Global equity index (long-term)</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>~7-9%</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
         <is>
-          <t>• Net gain rolls into Box 7.4 (kapitalvinst marknadsnoterade aktier/fonder)</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t>• ISA wrapper is irrelevant for Swedish tax — full gain taxable</t>
+          <t>Your Vanguard ISA return (2020-2025)</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>~10%/yr</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="16" t="inlineStr">
-        <is>
-          <t>• Capital losses elsewhere in 2025 can offset (100% against listed shares, 70% against other capital)</t>
-        </is>
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="n"/>
+      <c r="C49" s="14" t="n"/>
+      <c r="D49" s="14" t="n"/>
+      <c r="E49" s="14" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr">
+        <is>
+          <t>• 'Cash-on-cash' divides by equity, reflecting that you've only got ~£621k of own money in the flat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="inlineStr">
+        <is>
+          <t>• 'NOI yield' is pre-leverage — useful for comparing flats to other property investments before mortgage effects.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="inlineStr">
+        <is>
+          <t>• Total return reflects assumption that 2018-2025 CAGR continues forward. London may not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>• Post-CGT applies the implied 14.5% effective CGT rate (£24k on £165k gain) to forward appreciation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="inlineStr">
+        <is>
+          <t>• Excludes: voids, refurbishment beyond annual maintenance, mortgage refinance risk after May 2027 (rate may rise from 4.38%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>• Excludes: opportunity cost of equity. If £621k earned 5% in gilts = £31k/year passive — almost matches the steady-state cash yield.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>Zero-appreciation scenario (assume £0 capital growth)</t>
+        </is>
+      </c>
+      <c r="B58" s="14" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="14" t="n"/>
+      <c r="E58" s="14" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>(Conservative — reflects flat-to-down London market recent years)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="12" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="C61" s="12" t="inlineStr">
+        <is>
+          <t>% on value</t>
+        </is>
+      </c>
+      <c r="D61" s="12" t="inlineStr">
+        <is>
+          <t>% on equity</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Total return — 2025 cash only (with fee, 0% appreciation)</t>
+        </is>
+      </c>
+      <c r="B62">
+        <f>$B$34</f>
+        <v/>
+      </c>
+      <c r="C62" s="25">
+        <f>B62/$B$7</f>
+        <v/>
+      </c>
+      <c r="D62" s="25">
+        <f>B62/$B$9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="12" t="inlineStr">
+        <is>
+          <t>Total return — steady-state cash only (excl fee, 0% appreciation)</t>
+        </is>
+      </c>
+      <c r="B63" s="17">
+        <f>$B$36</f>
+        <v/>
+      </c>
+      <c r="C63" s="28">
+        <f>B63/$B$7</f>
+        <v/>
+      </c>
+      <c r="D63" s="28">
+        <f>B63/$B$9</f>
+        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7276,626 +7353,2776 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:G172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="4" min="1" max="1"/>
-    <col width="14" customWidth="1" style="4" min="2" max="2"/>
-    <col width="17" customWidth="1" style="4" min="3" max="3"/>
-    <col width="15" customWidth="1" style="4" min="4" max="4"/>
+    <col width="42" customWidth="1" style="4" min="1" max="1"/>
+    <col width="13" customWidth="1" style="4" min="2" max="2"/>
+    <col width="13" customWidth="1" style="4" min="3" max="3"/>
+    <col width="11" customWidth="1" style="4" min="4" max="4"/>
+    <col width="12" customWidth="1" style="4" min="5" max="5"/>
+    <col width="14" customWidth="1" style="4" min="6" max="6"/>
+    <col width="18" customWidth="1" style="4" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>76a Ingelow Road — Investment Yield Analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="16" t="inlineStr">
-        <is>
-          <t>Assuming gross-of-commission position for Swedish tax (£1,215 more conservative)</t>
+    <row r="1" ht="22" customHeight="1" s="4">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>Vanguard ISA — Capital Gains 2025 (genomsnittsmetoden, per fund)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Per Swedish tax law (44 kap. 14 § IL): omkostnadsbelopp = original acquisition cost in SEK at original-date FX. No rebasing on residency move.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>Inputs (edit to update yields)</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="n"/>
-      <c r="C4" s="14" t="n"/>
-      <c r="D4" s="14" t="n"/>
-      <c r="E4" s="14" t="n"/>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Genomsnittsmetoden applied per security. 4 funds traded: FTSE 100 UT Acc, VUSA, VMID, VERX. Pre-residency partial sale 15 Nov 2021 (FTSE 100) excluded.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Property purchase price (2018)</t>
-        </is>
-      </c>
-      <c r="B5" s="24" t="n">
-        <v>635000</v>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>FX = Riksbanken monthly Medel GBP/SEK (all verified 19 May 2026). Edit yellow cells to override.</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Years held (to 2025)</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Current property value</t>
-        </is>
-      </c>
-      <c r="B7" s="24" t="n">
-        <v>800000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Current mortgage outstanding (interest only)</t>
-        </is>
-      </c>
-      <c r="B8" s="24" t="n">
-        <v>178764.94</v>
-      </c>
-    </row>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Sources: Vanguard ISA VG0208845 transaction history PDFs (19 May 2026); Riksbanken sok-rantor-och-valutakurser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Equity in property (= value − mortgage)</t>
-        </is>
-      </c>
-      <c r="B9" s="15">
-        <f>$B$7-$B$8</f>
-        <v/>
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>K4 avsnitt A — rows to enter on Skatteverket e-tjänst</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Eventual CGT assumption (on current £165k appreciation)</t>
-        </is>
-      </c>
-      <c r="B10" s="24" t="n">
-        <v>24000</v>
+      <c r="A10" s="31" t="inlineStr">
+        <is>
+          <t>Antal</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Beteckning</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>Försäljningspris (SEK)</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="inlineStr">
+        <is>
+          <t>Omkostnadsbelopp (SEK)</t>
+        </is>
+      </c>
+      <c r="E10" s="31" t="inlineStr">
+        <is>
+          <t>Vinst (SEK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="32">
+        <f>$F$75</f>
+        <v/>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FTSE 100 Index Unit Trust Accumulation</t>
+        </is>
+      </c>
+      <c r="C11" s="33">
+        <f>$F$76</f>
+        <v/>
+      </c>
+      <c r="D11" s="33">
+        <f>$F$77</f>
+        <v/>
+      </c>
+      <c r="E11" s="33">
+        <f>$F$78</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Historical CAGR (from 2018 purchase)</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
+      <c r="A12" s="32">
+        <f>$F$115</f>
+        <v/>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 UCITS ETF — Distributing (VUSA)</t>
+        </is>
+      </c>
+      <c r="C12" s="33">
+        <f>$F$116</f>
+        <v/>
+      </c>
+      <c r="D12" s="33">
+        <f>$F$117</f>
+        <v/>
+      </c>
+      <c r="E12" s="33">
+        <f>$F$118</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Total appreciation (current − purchase)</t>
-        </is>
-      </c>
-      <c r="B13">
-        <f>$B$7-$B$5</f>
+      <c r="A13" s="32">
+        <f>$F$136</f>
+        <v/>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FTSE 250 UCITS ETF — Distributing (VMID)</t>
+        </is>
+      </c>
+      <c r="C13" s="33">
+        <f>$F$137</f>
+        <v/>
+      </c>
+      <c r="D13" s="33">
+        <f>$F$138</f>
+        <v/>
+      </c>
+      <c r="E13" s="33">
+        <f>$F$139</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Effective CGT rate on appreciation</t>
-        </is>
-      </c>
-      <c r="B14" s="25">
-        <f>$B$10/($B$7-$B$5)</f>
+      <c r="A14" s="32">
+        <f>$F$156</f>
+        <v/>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FTSE Developed Europe ex UK UCITS ETF — Distributing (VERX)</t>
+        </is>
+      </c>
+      <c r="C14" s="33">
+        <f>$F$157</f>
+        <v/>
+      </c>
+      <c r="D14" s="33">
+        <f>$F$158</f>
+        <v/>
+      </c>
+      <c r="E14" s="33">
+        <f>$F$159</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>CAGR (annualised)</t>
-        </is>
-      </c>
-      <c r="B15" s="26">
-        <f>($B$7/$B$5)^(1/$B$6)-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Forward annual appreciation (at CAGR × current value)</t>
-        </is>
-      </c>
-      <c r="B16">
-        <f>$B$7*$B$15</f>
-        <v/>
-      </c>
-    </row>
+      <c r="A15" s="34" t="n"/>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C15" s="36">
+        <f>SUM(C11:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="36">
+        <f>SUM(D11:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="37">
+        <f>SUM(E11:E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Forward appreciation AFTER CGT</t>
-        </is>
-      </c>
-      <c r="B17">
-        <f>$B$16*(1-$B$14)</f>
+      <c r="A17" s="30" t="inlineStr">
+        <is>
+          <t>Box 7.4 + Swedish tax</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Box 7.4 — Vinst fondandelar m.m. (SEK)</t>
+        </is>
+      </c>
+      <c r="C18" s="38">
+        <f>E15</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>Income statement 2025 (gross-of-commission Swedish, product fee in 2025)</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="14" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Swedish capital tax rate</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n">
+        <v>0.3</v>
+      </c>
     </row>
     <row r="20">
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Gross rental income (UK 25/26)</t>
-        </is>
-      </c>
-      <c r="B21">
-        <f>'Tax 25-26'!$B$16</f>
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Tax on Vanguard gain (SEK)</t>
+        </is>
+      </c>
+      <c r="C20" s="17">
+        <f>C18*C19</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Knight Frank commission</t>
-        </is>
-      </c>
-      <c r="B22">
-        <f>'Tax 25-26'!$B$17</f>
-        <v/>
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>FX rates — Riksbanken monthly Medel GBP/SEK (verified)</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Repairs &amp; maintenance</t>
-        </is>
-      </c>
-      <c r="B23">
-        <f>'Tax 25-26'!$B$19</f>
-        <v/>
-      </c>
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B23" s="31" t="inlineStr">
+        <is>
+          <t>FX rate (SEK per £1)</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="D23" s="39" t="n"/>
+      <c r="E23" s="39" t="n"/>
+      <c r="F23" s="39" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mortgage interest</t>
-        </is>
-      </c>
-      <c r="B24">
-        <f>-'Tax 25-26'!$B$23</f>
-        <v/>
+          <t>Sep 2020</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="n">
+        <v>11.45956</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mortgage product fee (one-off, 2025)</t>
-        </is>
-      </c>
-      <c r="B25">
-        <f>-'Tax 25-26'!$B$24</f>
-        <v/>
+          <t>Oct 2020</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="n">
+        <v>11.47127</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>UK tax on rental (net of finance credit)</t>
-        </is>
-      </c>
-      <c r="B26">
-        <f>-'Tax 25-26'!$B$32</f>
-        <v/>
+          <t>Nov 2020</t>
+        </is>
+      </c>
+      <c r="B26" s="40" t="n">
+        <v>11.41785</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Swedish tax on rental (gross-of-commission base, less FTC)</t>
-        </is>
-      </c>
-      <c r="B27">
-        <f>-((0.80*'Tax 25-26'!$B$37-'Tax 25-26'!$B$10/'Tax 25-26'!$B$4-'Tax 25-26'!$B$51)*0.30-'Tax 25-26'!$B$56)</f>
-        <v/>
+          <t>Dec 2020</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="n">
+        <v>11.23895</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr">
-        <is>
-          <t>Net cash income after all costs and tax (2025)</t>
-        </is>
-      </c>
-      <c r="B28" s="17">
-        <f>$B$21+$B$22+$B$23+$B$24+$B$25+$B$26+$B$27</f>
-        <v/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Jan 2021</t>
+        </is>
+      </c>
+      <c r="B28" s="40" t="n">
+        <v>11.31239</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="n">
+        <v>11.5525</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>Yield metrics</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="14" t="n"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="B30" s="40" t="n">
+        <v>11.83967</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="inlineStr">
-        <is>
-          <t>% on current value</t>
-        </is>
-      </c>
-      <c r="D31" s="12" t="inlineStr">
-        <is>
-          <t>% on equity</t>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Apr 2021</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="n">
+        <v>11.74595</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Gross yield (rent / value)</t>
-        </is>
-      </c>
-      <c r="B32">
-        <f>$B$21</f>
-        <v/>
-      </c>
-      <c r="C32" s="25">
-        <f>B32/$B$7</f>
-        <v/>
+          <t>May 2021</t>
+        </is>
+      </c>
+      <c r="B32" s="40" t="n">
+        <v>11.7571</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Net Operating Income (NOI — pre-leverage, pre-tax)</t>
-        </is>
-      </c>
-      <c r="B33">
-        <f>$B$21+$B$22+$B$23</f>
-        <v/>
-      </c>
-      <c r="C33" s="25">
-        <f>B33/$B$7</f>
-        <v/>
+          <t>Jun 2021</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="n">
+        <v>11.77512</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Net cash income (post all costs + tax, 2025)</t>
-        </is>
-      </c>
-      <c r="B34">
-        <f>$B$28</f>
-        <v/>
-      </c>
-      <c r="C34" s="25">
-        <f>B34/$B$7</f>
-        <v/>
-      </c>
-      <c r="D34" s="25">
-        <f>B34/$B$9</f>
-        <v/>
+          <t>Jul 2021</t>
+        </is>
+      </c>
+      <c r="B34" s="40" t="n">
+        <v>11.90743</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Aug 2021</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="n">
+        <v>11.97744</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Steady-state cash income (excl. product fee)</t>
-        </is>
-      </c>
-      <c r="B36">
-        <f>$B$28-$B$25</f>
-        <v/>
-      </c>
-      <c r="C36" s="25">
-        <f>B36/$B$7</f>
-        <v/>
-      </c>
-      <c r="D36" s="25">
-        <f>B36/$B$9</f>
-        <v/>
+          <t>Sep 2021</t>
+        </is>
+      </c>
+      <c r="B36" s="40" t="n">
+        <v>11.87028</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Oct 2021</t>
+        </is>
+      </c>
+      <c r="B37" s="40" t="n">
+        <v>11.86876</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Forward annual appreciation (CAGR × current value)</t>
-        </is>
-      </c>
-      <c r="B38">
-        <f>$B$16</f>
-        <v/>
-      </c>
-      <c r="C38" s="25">
-        <f>B38/$B$7</f>
-        <v/>
-      </c>
-      <c r="D38" s="25">
-        <f>B38/$B$9</f>
-        <v/>
+          <t>Nov 2021</t>
+        </is>
+      </c>
+      <c r="B38" s="40" t="n">
+        <v>11.84728</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>Total return — pre-CGT (steady cash + forward appreciation)</t>
-        </is>
-      </c>
-      <c r="B39" s="17">
-        <f>$B$36+$B$16</f>
-        <v/>
-      </c>
-      <c r="C39" s="27">
-        <f>B39/$B$7</f>
-        <v/>
-      </c>
-      <c r="D39" s="28">
-        <f>B39/$B$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="12" t="inlineStr">
-        <is>
-          <t>Total return — POST-CGT (steady cash + post-CGT appreciation)</t>
-        </is>
-      </c>
-      <c r="B40" s="17">
-        <f>$B$36+$B$17</f>
-        <v/>
-      </c>
-      <c r="C40" s="27">
-        <f>B40/$B$7</f>
-        <v/>
-      </c>
-      <c r="D40" s="28">
-        <f>B40/$B$9</f>
-        <v/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="B39" s="40" t="n">
+        <v>12.9485</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Riksbanken Medel</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="30" t="inlineStr">
+        <is>
+          <t>Fund: FTSE 100 Index Unit Trust Accumulation</t>
+        </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t>Benchmarks (rough reference)</t>
-        </is>
-      </c>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="14" t="n"/>
-      <c r="D42" s="14" t="n"/>
-      <c r="E42" s="14" t="n"/>
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>Buys</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t>UK 10-year gilts (risk-free)</t>
-        </is>
-      </c>
-      <c r="C43" s="16" t="inlineStr">
-        <is>
-          <t>~4-5%</t>
+      <c r="A43" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B43" s="31" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C43" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D43" s="31" t="inlineStr">
+        <is>
+          <t>FX month</t>
+        </is>
+      </c>
+      <c r="E43" s="31" t="inlineStr">
+        <is>
+          <t>FX rate</t>
+        </is>
+      </c>
+      <c r="F43" s="31" t="inlineStr">
+        <is>
+          <t>SEK cost</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="16" t="inlineStr">
-        <is>
-          <t>UK cash savings (instant access)</t>
-        </is>
-      </c>
-      <c r="C44" s="16" t="inlineStr">
-        <is>
-          <t>~4-5%</t>
-        </is>
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2020-09-25</t>
+        </is>
+      </c>
+      <c r="B44" s="32" t="n">
+        <v>0.9826</v>
+      </c>
+      <c r="C44" s="42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Sep 2020</t>
+        </is>
+      </c>
+      <c r="E44" s="43">
+        <f>$B$24</f>
+        <v/>
+      </c>
+      <c r="F44" s="33">
+        <f>C44*E44</f>
+        <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="16" t="inlineStr">
-        <is>
-          <t>UK FTSE 100 long-term nominal</t>
-        </is>
-      </c>
-      <c r="C45" s="16" t="inlineStr">
-        <is>
-          <t>~7-8%</t>
-        </is>
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2020-09-29</t>
+        </is>
+      </c>
+      <c r="B45" s="32" t="n">
+        <v>12.597</v>
+      </c>
+      <c r="C45" s="42" t="n">
+        <v>1254.41</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Sep 2020</t>
+        </is>
+      </c>
+      <c r="E45" s="43">
+        <f>$B$24</f>
+        <v/>
+      </c>
+      <c r="F45" s="33">
+        <f>C45*E45</f>
+        <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
-        <is>
-          <t>Global equity index (long-term)</t>
-        </is>
-      </c>
-      <c r="C46" s="16" t="inlineStr">
-        <is>
-          <t>~7-9%</t>
-        </is>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2020-11-02</t>
+        </is>
+      </c>
+      <c r="B46" s="32" t="n">
+        <v>1.0334</v>
+      </c>
+      <c r="C46" s="42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Nov 2020</t>
+        </is>
+      </c>
+      <c r="E46" s="43">
+        <f>$B$26</f>
+        <v/>
+      </c>
+      <c r="F46" s="33">
+        <f>C46*E46</f>
+        <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>Your Vanguard ISA return (2020-2025)</t>
-        </is>
-      </c>
-      <c r="C47" s="16" t="inlineStr">
-        <is>
-          <t>~10%/yr</t>
-        </is>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2020-12-01</t>
+        </is>
+      </c>
+      <c r="B47" s="32" t="n">
+        <v>0.9124</v>
+      </c>
+      <c r="C47" s="42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Dec 2020</t>
+        </is>
+      </c>
+      <c r="E47" s="43">
+        <f>$B$27</f>
+        <v/>
+      </c>
+      <c r="F47" s="33">
+        <f>C47*E47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2021-01-04</t>
+        </is>
+      </c>
+      <c r="B48" s="32" t="n">
+        <v>0.8808</v>
+      </c>
+      <c r="C48" s="42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Jan 2021</t>
+        </is>
+      </c>
+      <c r="E48" s="43">
+        <f>$B$28</f>
+        <v/>
+      </c>
+      <c r="F48" s="33">
+        <f>C48*E48</f>
+        <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="B49" s="14" t="n"/>
-      <c r="C49" s="14" t="n"/>
-      <c r="D49" s="14" t="n"/>
-      <c r="E49" s="14" t="n"/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2021-02-01</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="n">
+        <v>3.5798</v>
+      </c>
+      <c r="C49" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="E49" s="43">
+        <f>$B$29</f>
+        <v/>
+      </c>
+      <c r="F49" s="33">
+        <f>C49*E49</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="16" t="inlineStr">
-        <is>
-          <t>• 'Cash-on-cash' divides by equity, reflecting that you've only got ~£621k of own money in the flat.</t>
-        </is>
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2021-02-03</t>
+        </is>
+      </c>
+      <c r="B50" s="32" t="n">
+        <v>8.897600000000001</v>
+      </c>
+      <c r="C50" s="42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="E50" s="43">
+        <f>$B$29</f>
+        <v/>
+      </c>
+      <c r="F50" s="33">
+        <f>C50*E50</f>
+        <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="16" t="inlineStr">
-        <is>
-          <t>• 'NOI yield' is pre-leverage — useful for comparing flats to other property investments before mortgage effects.</t>
-        </is>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2021-02-04</t>
+        </is>
+      </c>
+      <c r="B51" s="32" t="n">
+        <v>8.897600000000001</v>
+      </c>
+      <c r="C51" s="42" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="E51" s="43">
+        <f>$B$29</f>
+        <v/>
+      </c>
+      <c r="F51" s="33">
+        <f>C51*E51</f>
+        <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="16" t="inlineStr">
-        <is>
-          <t>• Total return reflects assumption that 2018-2025 CAGR continues forward. London may not.</t>
-        </is>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2021-03-01</t>
+        </is>
+      </c>
+      <c r="B52" s="32" t="n">
+        <v>3.5005</v>
+      </c>
+      <c r="C52" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="E52" s="43">
+        <f>$B$30</f>
+        <v/>
+      </c>
+      <c r="F52" s="33">
+        <f>C52*E52</f>
+        <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>• Post-CGT applies the implied 14.5% effective CGT rate (£24k on £165k gain) to forward appreciation.</t>
-        </is>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2021-03-05</t>
+        </is>
+      </c>
+      <c r="B53" s="32" t="n">
+        <v>4.3373</v>
+      </c>
+      <c r="C53" s="42" t="n">
+        <v>500</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="E53" s="43">
+        <f>$B$30</f>
+        <v/>
+      </c>
+      <c r="F53" s="33">
+        <f>C53*E53</f>
+        <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="16" t="inlineStr">
-        <is>
-          <t>• Excludes: voids, refurbishment beyond annual maintenance, mortgage refinance risk after May 2027 (rate may rise from 4.38%).</t>
-        </is>
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2021-04-01</t>
+        </is>
+      </c>
+      <c r="B54" s="32" t="n">
+        <v>3.4025</v>
+      </c>
+      <c r="C54" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Apr 2021</t>
+        </is>
+      </c>
+      <c r="E54" s="43">
+        <f>$B$31</f>
+        <v/>
+      </c>
+      <c r="F54" s="33">
+        <f>C54*E54</f>
+        <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="16" t="inlineStr">
-        <is>
-          <t>• Excludes: opportunity cost of equity. If £621k earned 5% in gilts = £31k/year passive — almost matches the steady-state cash yield.</t>
-        </is>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2021-04-20</t>
+        </is>
+      </c>
+      <c r="B55" s="32" t="n">
+        <v>6.2246</v>
+      </c>
+      <c r="C55" s="42" t="n">
+        <v>750</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Apr 2021</t>
+        </is>
+      </c>
+      <c r="E55" s="43">
+        <f>$B$31</f>
+        <v/>
+      </c>
+      <c r="F55" s="33">
+        <f>C55*E55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2021-05-04</t>
+        </is>
+      </c>
+      <c r="B56" s="32" t="n">
+        <v>3.319</v>
+      </c>
+      <c r="C56" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>May 2021</t>
+        </is>
+      </c>
+      <c r="E56" s="43">
+        <f>$B$32</f>
+        <v/>
+      </c>
+      <c r="F56" s="33">
+        <f>C56*E56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2021-06-01</t>
+        </is>
+      </c>
+      <c r="B57" s="32" t="n">
+        <v>3.2354</v>
+      </c>
+      <c r="C57" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Jun 2021</t>
+        </is>
+      </c>
+      <c r="E57" s="43">
+        <f>$B$33</f>
+        <v/>
+      </c>
+      <c r="F57" s="33">
+        <f>C57*E57</f>
+        <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="13" t="inlineStr">
-        <is>
-          <t>Zero-appreciation scenario (assume £0 capital growth)</t>
-        </is>
-      </c>
-      <c r="B58" s="14" t="n"/>
-      <c r="C58" s="14" t="n"/>
-      <c r="D58" s="14" t="n"/>
-      <c r="E58" s="14" t="n"/>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2021-07-01</t>
+        </is>
+      </c>
+      <c r="B58" s="32" t="n">
+        <v>3.1929</v>
+      </c>
+      <c r="C58" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Jul 2021</t>
+        </is>
+      </c>
+      <c r="E58" s="43">
+        <f>$B$34</f>
+        <v/>
+      </c>
+      <c r="F58" s="33">
+        <f>C58*E58</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="16" t="inlineStr">
-        <is>
-          <t>(Conservative — reflects flat-to-down London market recent years)</t>
-        </is>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2021-08-02</t>
+        </is>
+      </c>
+      <c r="B59" s="32" t="n">
+        <v>3.2245</v>
+      </c>
+      <c r="C59" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Aug 2021</t>
+        </is>
+      </c>
+      <c r="E59" s="43">
+        <f>$B$35</f>
+        <v/>
+      </c>
+      <c r="F59" s="33">
+        <f>C59*E59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2021-08-29</t>
+        </is>
+      </c>
+      <c r="B60" s="32" t="n">
+        <v>1.591</v>
+      </c>
+      <c r="C60" s="42" t="n">
+        <v>200</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Aug 2021</t>
+        </is>
+      </c>
+      <c r="E60" s="43">
+        <f>$B$35</f>
+        <v/>
+      </c>
+      <c r="F60" s="33">
+        <f>C60*E60</f>
+        <v/>
       </c>
     </row>
     <row r="61">
-      <c r="B61" s="12" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="C61" s="12" t="inlineStr">
-        <is>
-          <t>% on value</t>
-        </is>
-      </c>
-      <c r="D61" s="12" t="inlineStr">
-        <is>
-          <t>% on equity</t>
-        </is>
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2021-09-01</t>
+        </is>
+      </c>
+      <c r="B61" s="32" t="n">
+        <v>3.1681</v>
+      </c>
+      <c r="C61" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Sep 2021</t>
+        </is>
+      </c>
+      <c r="E61" s="43">
+        <f>$B$36</f>
+        <v/>
+      </c>
+      <c r="F61" s="33">
+        <f>C61*E61</f>
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Total return — 2025 cash only (with fee, 0% appreciation)</t>
-        </is>
-      </c>
-      <c r="B62">
+          <t>2021-10-01</t>
+        </is>
+      </c>
+      <c r="B62" s="32" t="n">
+        <v>3.2146</v>
+      </c>
+      <c r="C62" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Oct 2021</t>
+        </is>
+      </c>
+      <c r="E62" s="43">
+        <f>$B$37</f>
+        <v/>
+      </c>
+      <c r="F62" s="33">
+        <f>C62*E62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2021-11-01</t>
+        </is>
+      </c>
+      <c r="B63" s="32" t="n">
+        <v>3.0974</v>
+      </c>
+      <c r="C63" s="42" t="n">
+        <v>400</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Nov 2021</t>
+        </is>
+      </c>
+      <c r="E63" s="43">
+        <f>$B$38</f>
+        <v/>
+      </c>
+      <c r="F63" s="33">
+        <f>C63*E63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="35" t="inlineStr">
+        <is>
+          <t>Total buys</t>
+        </is>
+      </c>
+      <c r="B64" s="44">
+        <f>SUM(B44:B63)</f>
+        <v/>
+      </c>
+      <c r="C64" s="45">
+        <f>SUM(C44:C63)</f>
+        <v/>
+      </c>
+      <c r="D64" s="46" t="n"/>
+      <c r="E64" s="46" t="n"/>
+      <c r="F64" s="36">
+        <f>SUM(F44:F63)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="12" t="inlineStr">
+        <is>
+          <t>Average cost per unit (SEK)</t>
+        </is>
+      </c>
+      <c r="F65" s="33">
+        <f>$F$64/$B$64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="41" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B68" s="31" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C68" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D68" s="31" t="inlineStr">
+        <is>
+          <t>FX month</t>
+        </is>
+      </c>
+      <c r="E68" s="31" t="inlineStr">
+        <is>
+          <t>FX rate</t>
+        </is>
+      </c>
+      <c r="F68" s="31" t="inlineStr"/>
+      <c r="G68" s="31" t="inlineStr">
+        <is>
+          <t>Swedish 2025?</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="47" t="inlineStr">
+        <is>
+          <t>2021-11-15</t>
+        </is>
+      </c>
+      <c r="B69" s="48" t="n">
+        <v>5.0134</v>
+      </c>
+      <c r="C69" s="49" t="n">
+        <v>657.26</v>
+      </c>
+      <c r="D69" s="47" t="inlineStr">
+        <is>
+          <t>Nov 2021</t>
+        </is>
+      </c>
+      <c r="E69" s="50">
+        <f>$B$38</f>
+        <v/>
+      </c>
+      <c r="F69" s="51">
+        <f>C69*E69</f>
+        <v/>
+      </c>
+      <c r="G69" s="47" t="inlineStr">
+        <is>
+          <t>No — pre-residency</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2025-06-09</t>
+        </is>
+      </c>
+      <c r="B70" s="32" t="n">
+        <v>41.7177</v>
+      </c>
+      <c r="C70" s="42" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="E70" s="43">
+        <f>$B$39</f>
+        <v/>
+      </c>
+      <c r="F70" s="33">
+        <f>C70*E70</f>
+        <v/>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2025-06-17</t>
+        </is>
+      </c>
+      <c r="B71" s="32" t="n">
+        <v>32.5579</v>
+      </c>
+      <c r="C71" s="42" t="n">
+        <v>5861.72</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="E71" s="43">
+        <f>$B$39</f>
+        <v/>
+      </c>
+      <c r="F71" s="33">
+        <f>C71*E71</f>
+        <v/>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="35" t="inlineStr">
+        <is>
+          <t>Swedish 2025 sale total</t>
+        </is>
+      </c>
+      <c r="B72" s="44">
+        <f>B70+B71</f>
+        <v/>
+      </c>
+      <c r="C72" s="46" t="n"/>
+      <c r="D72" s="46" t="n"/>
+      <c r="E72" s="46" t="n"/>
+      <c r="F72" s="36">
+        <f>F70+F71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="41" t="inlineStr">
+        <is>
+          <t>K4 calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Units sold in 2025 (Antal)</t>
+        </is>
+      </c>
+      <c r="F75" s="32">
+        <f>$B$72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Försäljningspris (SEK)</t>
+        </is>
+      </c>
+      <c r="F76" s="33">
+        <f>$F$72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Omkostnadsbelopp = units × avg cost (SEK)</t>
+        </is>
+      </c>
+      <c r="F77" s="33">
+        <f>$F$75*$F$65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="inlineStr">
+        <is>
+          <t>Vinst (SEK)</t>
+        </is>
+      </c>
+      <c r="F78" s="38">
+        <f>$F$76-$F$77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="30" t="inlineStr">
+        <is>
+          <t>Fund: S&amp;P 500 UCITS ETF — Distributing (VUSA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="41" t="inlineStr">
+        <is>
+          <t>Buys</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B83" s="31" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C83" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D83" s="31" t="inlineStr">
+        <is>
+          <t>FX month</t>
+        </is>
+      </c>
+      <c r="E83" s="31" t="inlineStr">
+        <is>
+          <t>FX rate</t>
+        </is>
+      </c>
+      <c r="F83" s="31" t="inlineStr">
+        <is>
+          <t>SEK cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2020-09-25</t>
+        </is>
+      </c>
+      <c r="B84" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" s="42" t="n">
+        <v>98.25</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Sep 2020</t>
+        </is>
+      </c>
+      <c r="E84" s="43">
+        <f>$B$24</f>
+        <v/>
+      </c>
+      <c r="F84" s="33">
+        <f>C84*E84</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2020-09-29</t>
+        </is>
+      </c>
+      <c r="B85" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="C85" s="42" t="n">
+        <v>1244.85</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Sep 2020</t>
+        </is>
+      </c>
+      <c r="E85" s="43">
+        <f>$B$24</f>
+        <v/>
+      </c>
+      <c r="F85" s="33">
+        <f>C85*E85</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2020-11-02</t>
+        </is>
+      </c>
+      <c r="B86" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C86" s="42" t="n">
+        <v>97.45999999999999</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Nov 2020</t>
+        </is>
+      </c>
+      <c r="E86" s="43">
+        <f>$B$26</f>
+        <v/>
+      </c>
+      <c r="F86" s="33">
+        <f>C86*E86</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2020-12-01</t>
+        </is>
+      </c>
+      <c r="B87" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" s="42" t="n">
+        <v>51.99</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Dec 2020</t>
+        </is>
+      </c>
+      <c r="E87" s="43">
+        <f>$B$27</f>
+        <v/>
+      </c>
+      <c r="F87" s="33">
+        <f>C87*E87</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2020-12-01</t>
+        </is>
+      </c>
+      <c r="B88" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C88" s="42" t="n">
+        <v>52.09</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Dec 2020</t>
+        </is>
+      </c>
+      <c r="E88" s="43">
+        <f>$B$27</f>
+        <v/>
+      </c>
+      <c r="F88" s="33">
+        <f>C88*E88</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2021-01-04</t>
+        </is>
+      </c>
+      <c r="B89" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C89" s="42" t="n">
+        <v>52.42</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Jan 2021</t>
+        </is>
+      </c>
+      <c r="E89" s="43">
+        <f>$B$28</f>
+        <v/>
+      </c>
+      <c r="F89" s="33">
+        <f>C89*E89</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2021-01-06</t>
+        </is>
+      </c>
+      <c r="B90" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" s="42" t="n">
+        <v>51.63</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Jan 2021</t>
+        </is>
+      </c>
+      <c r="E90" s="43">
+        <f>$B$28</f>
+        <v/>
+      </c>
+      <c r="F90" s="33">
+        <f>C90*E90</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2021-02-01</t>
+        </is>
+      </c>
+      <c r="B91" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C91" s="42" t="n">
+        <v>362.81</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="E91" s="43">
+        <f>$B$29</f>
+        <v/>
+      </c>
+      <c r="F91" s="33">
+        <f>C91*E91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2021-02-03</t>
+        </is>
+      </c>
+      <c r="B92" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="C92" s="42" t="n">
+        <v>963.86</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="E92" s="43">
+        <f>$B$29</f>
+        <v/>
+      </c>
+      <c r="F92" s="33">
+        <f>C92*E92</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2021-02-04</t>
+        </is>
+      </c>
+      <c r="B93" s="32" t="n">
+        <v>18</v>
+      </c>
+      <c r="C93" s="42" t="n">
+        <v>963.86</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="E93" s="43">
+        <f>$B$29</f>
+        <v/>
+      </c>
+      <c r="F93" s="33">
+        <f>C93*E93</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2021-03-01</t>
+        </is>
+      </c>
+      <c r="B94" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C94" s="42" t="n">
+        <v>367.71</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="E94" s="43">
+        <f>$B$30</f>
+        <v/>
+      </c>
+      <c r="F94" s="33">
+        <f>C94*E94</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2021-03-05</t>
+        </is>
+      </c>
+      <c r="B95" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C95" s="42" t="n">
+        <v>465.14</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="E95" s="43">
+        <f>$B$30</f>
+        <v/>
+      </c>
+      <c r="F95" s="33">
+        <f>C95*E95</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2021-03-22</t>
+        </is>
+      </c>
+      <c r="B96" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C96" s="42" t="n">
+        <v>384.29</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="E96" s="43">
+        <f>$B$30</f>
+        <v/>
+      </c>
+      <c r="F96" s="33">
+        <f>C96*E96</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2021-04-20</t>
+        </is>
+      </c>
+      <c r="B97" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C97" s="42" t="n">
+        <v>731.53</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Apr 2021</t>
+        </is>
+      </c>
+      <c r="E97" s="43">
+        <f>$B$31</f>
+        <v/>
+      </c>
+      <c r="F97" s="33">
+        <f>C97*E97</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2021-04-21</t>
+        </is>
+      </c>
+      <c r="B98" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C98" s="42" t="n">
+        <v>343.56</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Apr 2021</t>
+        </is>
+      </c>
+      <c r="E98" s="43">
+        <f>$B$31</f>
+        <v/>
+      </c>
+      <c r="F98" s="33">
+        <f>C98*E98</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2021-05-19</t>
+        </is>
+      </c>
+      <c r="B99" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C99" s="42" t="n">
+        <v>395.8</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>May 2021</t>
+        </is>
+      </c>
+      <c r="E99" s="43">
+        <f>$B$32</f>
+        <v/>
+      </c>
+      <c r="F99" s="33">
+        <f>C99*E99</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2021-06-21</t>
+        </is>
+      </c>
+      <c r="B100" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C100" s="42" t="n">
+        <v>355.37</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Jun 2021</t>
+        </is>
+      </c>
+      <c r="E100" s="43">
+        <f>$B$33</f>
+        <v/>
+      </c>
+      <c r="F100" s="33">
+        <f>C100*E100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2021-07-21</t>
+        </is>
+      </c>
+      <c r="B101" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C101" s="42" t="n">
+        <v>361.88</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Jul 2021</t>
+        </is>
+      </c>
+      <c r="E101" s="43">
         <f>$B$34</f>
         <v/>
       </c>
-      <c r="C62" s="25">
-        <f>B62/$B$7</f>
-        <v/>
-      </c>
-      <c r="D62" s="25">
-        <f>B62/$B$9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="12" t="inlineStr">
-        <is>
-          <t>Total return — steady-state cash only (excl fee, 0% appreciation)</t>
-        </is>
-      </c>
-      <c r="B63" s="17">
+      <c r="F101" s="33">
+        <f>C101*E101</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2021-08-19</t>
+        </is>
+      </c>
+      <c r="B102" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C102" s="42" t="n">
+        <v>376.08</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Aug 2021</t>
+        </is>
+      </c>
+      <c r="E102" s="43">
+        <f>$B$35</f>
+        <v/>
+      </c>
+      <c r="F102" s="33">
+        <f>C102*E102</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2021-09-21</t>
+        </is>
+      </c>
+      <c r="B103" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C103" s="42" t="n">
+        <v>361.55</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Sep 2021</t>
+        </is>
+      </c>
+      <c r="E103" s="43">
         <f>$B$36</f>
         <v/>
       </c>
-      <c r="C63" s="28">
-        <f>B63/$B$7</f>
-        <v/>
-      </c>
-      <c r="D63" s="28">
-        <f>B63/$B$9</f>
-        <v/>
+      <c r="F103" s="33">
+        <f>C103*E103</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2021-10-20</t>
+        </is>
+      </c>
+      <c r="B104" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C104" s="42" t="n">
+        <v>385.28</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Oct 2021</t>
+        </is>
+      </c>
+      <c r="E104" s="43">
+        <f>$B$37</f>
+        <v/>
+      </c>
+      <c r="F104" s="33">
+        <f>C104*E104</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="35" t="inlineStr">
+        <is>
+          <t>Total buys</t>
+        </is>
+      </c>
+      <c r="B105" s="44">
+        <f>SUM(B84:B104)</f>
+        <v/>
+      </c>
+      <c r="C105" s="45">
+        <f>SUM(C84:C104)</f>
+        <v/>
+      </c>
+      <c r="D105" s="46" t="n"/>
+      <c r="E105" s="46" t="n"/>
+      <c r="F105" s="36">
+        <f>SUM(F84:F104)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="12" t="inlineStr">
+        <is>
+          <t>Average cost per unit (SEK)</t>
+        </is>
+      </c>
+      <c r="F106" s="33">
+        <f>$F$105/$B$105</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="41" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B109" s="31" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C109" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D109" s="31" t="inlineStr">
+        <is>
+          <t>FX month</t>
+        </is>
+      </c>
+      <c r="E109" s="31" t="inlineStr">
+        <is>
+          <t>FX rate</t>
+        </is>
+      </c>
+      <c r="F109" s="31" t="inlineStr"/>
+      <c r="G109" s="31" t="inlineStr">
+        <is>
+          <t>Swedish 2025?</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2025-06-09</t>
+        </is>
+      </c>
+      <c r="B110" s="32" t="n">
+        <v>90</v>
+      </c>
+      <c r="C110" s="42" t="n">
+        <v>7544.99</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="E110" s="43">
+        <f>$B$39</f>
+        <v/>
+      </c>
+      <c r="F110" s="33">
+        <f>C110*E110</f>
+        <v/>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2025-06-17</t>
+        </is>
+      </c>
+      <c r="B111" s="32" t="n">
+        <v>65</v>
+      </c>
+      <c r="C111" s="42" t="n">
+        <v>5456.78</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="E111" s="43">
+        <f>$B$39</f>
+        <v/>
+      </c>
+      <c r="F111" s="33">
+        <f>C111*E111</f>
+        <v/>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="35" t="inlineStr">
+        <is>
+          <t>Swedish 2025 sale total</t>
+        </is>
+      </c>
+      <c r="B112" s="44">
+        <f>B110+B111</f>
+        <v/>
+      </c>
+      <c r="C112" s="46" t="n"/>
+      <c r="D112" s="46" t="n"/>
+      <c r="E112" s="46" t="n"/>
+      <c r="F112" s="36">
+        <f>F110+F111</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="41" t="inlineStr">
+        <is>
+          <t>K4 calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Units sold in 2025 (Antal)</t>
+        </is>
+      </c>
+      <c r="F115" s="32">
+        <f>$B$112</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Försäljningspris (SEK)</t>
+        </is>
+      </c>
+      <c r="F116" s="33">
+        <f>$F$112</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Omkostnadsbelopp = units × avg cost (SEK)</t>
+        </is>
+      </c>
+      <c r="F117" s="33">
+        <f>$F$115*$F$106</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="12" t="inlineStr">
+        <is>
+          <t>Vinst (SEK)</t>
+        </is>
+      </c>
+      <c r="F118" s="38">
+        <f>$F$116-$F$117</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="30" t="inlineStr">
+        <is>
+          <t>Fund: FTSE 250 UCITS ETF — Distributing (VMID)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="41" t="inlineStr">
+        <is>
+          <t>Buys</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B123" s="31" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C123" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D123" s="31" t="inlineStr">
+        <is>
+          <t>FX month</t>
+        </is>
+      </c>
+      <c r="E123" s="31" t="inlineStr">
+        <is>
+          <t>FX rate</t>
+        </is>
+      </c>
+      <c r="F123" s="31" t="inlineStr">
+        <is>
+          <t>SEK cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2021-02-10</t>
+        </is>
+      </c>
+      <c r="B124" s="32" t="n">
+        <v>30</v>
+      </c>
+      <c r="C124" s="42" t="n">
+        <v>993.41</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="E124" s="43">
+        <f>$B$29</f>
+        <v/>
+      </c>
+      <c r="F124" s="33">
+        <f>C124*E124</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2021-03-05</t>
+        </is>
+      </c>
+      <c r="B125" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C125" s="42" t="n">
+        <v>233.18</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="E125" s="43">
+        <f>$B$30</f>
+        <v/>
+      </c>
+      <c r="F125" s="33">
+        <f>C125*E125</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2021-04-20</t>
+        </is>
+      </c>
+      <c r="B126" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C126" s="42" t="n">
+        <v>277.38</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Apr 2021</t>
+        </is>
+      </c>
+      <c r="E126" s="43">
+        <f>$B$31</f>
+        <v/>
+      </c>
+      <c r="F126" s="33">
+        <f>C126*E126</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="35" t="inlineStr">
+        <is>
+          <t>Total buys</t>
+        </is>
+      </c>
+      <c r="B127" s="44">
+        <f>SUM(B124:B126)</f>
+        <v/>
+      </c>
+      <c r="C127" s="45">
+        <f>SUM(C124:C126)</f>
+        <v/>
+      </c>
+      <c r="D127" s="46" t="n"/>
+      <c r="E127" s="46" t="n"/>
+      <c r="F127" s="36">
+        <f>SUM(F124:F126)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="12" t="inlineStr">
+        <is>
+          <t>Average cost per unit (SEK)</t>
+        </is>
+      </c>
+      <c r="F128" s="33">
+        <f>$F$127/$B$127</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="41" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B131" s="31" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C131" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D131" s="31" t="inlineStr">
+        <is>
+          <t>FX month</t>
+        </is>
+      </c>
+      <c r="E131" s="31" t="inlineStr">
+        <is>
+          <t>FX rate</t>
+        </is>
+      </c>
+      <c r="F131" s="31" t="inlineStr"/>
+      <c r="G131" s="31" t="inlineStr">
+        <is>
+          <t>Swedish 2025?</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="B132" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="C132" s="42" t="n">
+        <v>1457.21</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="E132" s="43">
+        <f>$B$39</f>
+        <v/>
+      </c>
+      <c r="F132" s="33">
+        <f>C132*E132</f>
+        <v/>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="35" t="inlineStr">
+        <is>
+          <t>Swedish 2025 sale total</t>
+        </is>
+      </c>
+      <c r="B133" s="44">
+        <f>B132</f>
+        <v/>
+      </c>
+      <c r="C133" s="46" t="n"/>
+      <c r="D133" s="46" t="n"/>
+      <c r="E133" s="46" t="n"/>
+      <c r="F133" s="36">
+        <f>F132</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="41" t="inlineStr">
+        <is>
+          <t>K4 calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Units sold in 2025 (Antal)</t>
+        </is>
+      </c>
+      <c r="F136" s="32">
+        <f>$B$133</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Försäljningspris (SEK)</t>
+        </is>
+      </c>
+      <c r="F137" s="33">
+        <f>$F$133</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Omkostnadsbelopp = units × avg cost (SEK)</t>
+        </is>
+      </c>
+      <c r="F138" s="33">
+        <f>$F$136*$F$128</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="12" t="inlineStr">
+        <is>
+          <t>Vinst (SEK)</t>
+        </is>
+      </c>
+      <c r="F139" s="38">
+        <f>$F$137-$F$138</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="30" t="inlineStr">
+        <is>
+          <t>Fund: FTSE Developed Europe ex UK UCITS ETF — Distributing (VERX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="41" t="inlineStr">
+        <is>
+          <t>Buys</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B144" s="31" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C144" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D144" s="31" t="inlineStr">
+        <is>
+          <t>FX month</t>
+        </is>
+      </c>
+      <c r="E144" s="31" t="inlineStr">
+        <is>
+          <t>FX rate</t>
+        </is>
+      </c>
+      <c r="F144" s="31" t="inlineStr">
+        <is>
+          <t>SEK cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2021-02-10</t>
+        </is>
+      </c>
+      <c r="B145" s="32" t="n">
+        <v>34</v>
+      </c>
+      <c r="C145" s="42" t="n">
+        <v>974.39</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="E145" s="43">
+        <f>$B$29</f>
+        <v/>
+      </c>
+      <c r="F145" s="33">
+        <f>C145*E145</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2021-03-14</t>
+        </is>
+      </c>
+      <c r="B146" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C146" s="42" t="n">
+        <v>232.16</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="E146" s="43">
+        <f>$B$30</f>
+        <v/>
+      </c>
+      <c r="F146" s="33">
+        <f>C146*E146</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="35" t="inlineStr">
+        <is>
+          <t>Total buys</t>
+        </is>
+      </c>
+      <c r="B147" s="44">
+        <f>SUM(B145:B146)</f>
+        <v/>
+      </c>
+      <c r="C147" s="45">
+        <f>SUM(C145:C146)</f>
+        <v/>
+      </c>
+      <c r="D147" s="46" t="n"/>
+      <c r="E147" s="46" t="n"/>
+      <c r="F147" s="36">
+        <f>SUM(F145:F146)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
+        <is>
+          <t>Average cost per unit (SEK)</t>
+        </is>
+      </c>
+      <c r="F148" s="33">
+        <f>$F$147/$B$147</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="41" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B151" s="31" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C151" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D151" s="31" t="inlineStr">
+        <is>
+          <t>FX month</t>
+        </is>
+      </c>
+      <c r="E151" s="31" t="inlineStr">
+        <is>
+          <t>FX rate</t>
+        </is>
+      </c>
+      <c r="F151" s="31" t="inlineStr"/>
+      <c r="G151" s="31" t="inlineStr">
+        <is>
+          <t>Swedish 2025?</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2025-06-05</t>
+        </is>
+      </c>
+      <c r="B152" s="32" t="n">
+        <v>42</v>
+      </c>
+      <c r="C152" s="42" t="n">
+        <v>1541.25</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="E152" s="43">
+        <f>$B$39</f>
+        <v/>
+      </c>
+      <c r="F152" s="33">
+        <f>C152*E152</f>
+        <v/>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="35" t="inlineStr">
+        <is>
+          <t>Swedish 2025 sale total</t>
+        </is>
+      </c>
+      <c r="B153" s="44">
+        <f>B152</f>
+        <v/>
+      </c>
+      <c r="C153" s="46" t="n"/>
+      <c r="D153" s="46" t="n"/>
+      <c r="E153" s="46" t="n"/>
+      <c r="F153" s="36">
+        <f>F152</f>
+        <v/>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="41" t="inlineStr">
+        <is>
+          <t>K4 calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Units sold in 2025 (Antal)</t>
+        </is>
+      </c>
+      <c r="F156" s="32">
+        <f>$B$153</f>
+        <v/>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Försäljningspris (SEK)</t>
+        </is>
+      </c>
+      <c r="F157" s="33">
+        <f>$F$153</f>
+        <v/>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Omkostnadsbelopp = units × avg cost (SEK)</t>
+        </is>
+      </c>
+      <c r="F158" s="33">
+        <f>$F$156*$F$148</f>
+        <v/>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="12" t="inlineStr">
+        <is>
+          <t>Vinst (SEK)</t>
+        </is>
+      </c>
+      <c r="F159" s="38">
+        <f>$F$157-$F$158</f>
+        <v/>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="30" t="inlineStr">
+        <is>
+          <t>Excluded — FTSE Developed Europe ex-U.K. Equity Index Fund (Accumulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="16" t="inlineStr">
+        <is>
+          <t>Bought 05 Mar 2021 (£250, 0.8601 units) and sold 14 Mar 2021 (£259.10, 0.8601 units). Both pre-Swedish-residency. Not on Swedish return.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="30" t="inlineStr">
+        <is>
+          <t>Method &amp; references</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="16" t="inlineStr">
+        <is>
+          <t>• Genomsnittsmetoden applied per security (ISIN). Each fund has its own omkostnadsbelopp pool.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="16" t="inlineStr">
+        <is>
+          <t>• Each buy converted to SEK at Riksbanken monthly Medel GBP/SEK for the buy month. Sale proceeds converted at the sale month's Medel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="16" t="inlineStr">
+        <is>
+          <t>• FTSE 100 had a pre-residency partial sale on 15 Nov 2021 (5.0134 units, £657.26). That sale is not on the Swedish return; it just reduces the unit pool. The remaining units carry the same average cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="16" t="inlineStr">
+        <is>
+          <t>• Swedish tax resident from 25 Nov 2021. All buys completed by 1 Nov 2021 — all pre-residency, but pre-residency buys still constitute the omkostnadsbelopp under Swedish rules (no rebasing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="16" t="inlineStr">
+        <is>
+          <t>• ISA wrapper is irrelevant for Swedish tax — the full gain is taxable. Lossen från 2025 can offset (100% mot marknadsnoterade aktier/fonder; 70% mot annan kapital).</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="16" t="inlineStr">
+        <is>
+          <t>• File K4 avsnitt A with the 4 rows above. Box 7.4 = sum of the 4 vinst figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="16" t="inlineStr">
+        <is>
+          <t>• Sources: 44 kap. 14 § Inkomstskattelagen; Skatteverket 'Utländsk valuta'; Vanguard ISA transaction PDFs (19 May 2026); Riksbanken sok-rantor-och-valutakurser.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+  <mergeCells count="34">
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A172:F172"/>
+    <mergeCell ref="A108:F108"/>
+    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="A163:F163"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A150:F150"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A135:F135"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A122:F122"/>
+    <mergeCell ref="A171:F171"/>
+    <mergeCell ref="A165:F165"/>
+    <mergeCell ref="A81:F81"/>
+    <mergeCell ref="A170:F170"/>
+    <mergeCell ref="A121:F121"/>
+    <mergeCell ref="A155:F155"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A67:F67"/>
+    <mergeCell ref="A167:F167"/>
+    <mergeCell ref="A143:F143"/>
+    <mergeCell ref="A130:F130"/>
+    <mergeCell ref="A114:F114"/>
+    <mergeCell ref="A166:F166"/>
+    <mergeCell ref="A142:F142"/>
+    <mergeCell ref="A82:F82"/>
+    <mergeCell ref="A169:F169"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A168:F168"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="A162:F162"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Post-filing canonical record: rebuild guide.md + docx, add Submissions xlsx tab, archive Vanguard PDFs, add 2026 checklist
</commit_message>
<xml_diff>
--- a/projects/uk-rental/Tax_Return.xlsx
+++ b/projects/uk-rental/Tax_Return.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2800" yWindow="1540" windowWidth="28040" windowHeight="17180" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="76A Ingelow Road" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Santander" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tax 24-25" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Tax 25-26" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="HSBC Interest" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Yield Analysis" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Capital Gains 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Submissions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="76A Ingelow Road" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Santander" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tax 24-25" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tax 25-26" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HSBC Interest" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yield Analysis" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capital Gains 2025" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -27,7 +28,7 @@
     <numFmt numFmtId="166" formatCode="0.0000"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -91,8 +92,12 @@
       <i val="1"/>
       <color rgb="00808080"/>
     </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -154,6 +159,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -168,7 +178,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,6 +233,11 @@
     <xf numFmtId="4" fontId="12" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="12" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="12" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -621,6 +636,864 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="4" min="1" max="1"/>
+    <col width="50" customWidth="1" style="4" min="2" max="2"/>
+    <col width="18" customWidth="1" style="4" min="3" max="3"/>
+    <col width="18" customWidth="1" style="4" min="4" max="4"/>
+    <col width="50" customWidth="1" style="4" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="4">
+      <c r="A1" s="52" t="inlineStr">
+        <is>
+          <t>Tax Returns 2025 — Submission Record</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Both returns submitted 2026-05-19. This tab is the single source of truth — all other tabs are working calcs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>Submission references</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>Jurisdiction</t>
+        </is>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>Form</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>Date/time</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="E5" s="31" t="inlineStr">
+        <is>
+          <t>Receipt file</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>HMRC (UK)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SA100 + SA105 2025/26</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-05-19 07:38 GMT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2605755020</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>UK_Tax_Return_2025-26_filed.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Skatteverket (Sweden)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>INK1 + K4 avsnitt A 2025</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-05-19 10:14 CEST</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>20260519101426199209225011262906</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Swedish_Tax_Return_2025_kvittens.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>Swedish INK1 2025 — submitted values</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="31" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="inlineStr">
+        <is>
+          <t>SEK</t>
+        </is>
+      </c>
+      <c r="D10" s="31" t="inlineStr"/>
+      <c r="E10" s="31" t="inlineStr">
+        <is>
+          <t>Working source</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Lön, förmåner (förtryckt)</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="n">
+        <v>705810</v>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>Skatteverket förtryckt (KU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Småhus/ägarlägenhet 0,75 % (Swedish property, sold 2026)</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="n">
+        <v>671600</v>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Skatteverket förtryckt (taxeringsvärde)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Schablonintäkter (förtryckt)</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="n">
+        <v>18360</v>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Förtryckt ISK/fond</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>7.2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Ränteinkomster (322 förtryckt + 2,730 HSBC UK)</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="n">
+        <v>3052</v>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>HSBC Interest tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Överskott vid uthyrning av privatbostad</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="n">
+        <v>310434</v>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Tax 25-26 tab; Knight Frank 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Vinst fondandelar (Vanguard ISA, K4)</t>
+        </is>
+      </c>
+      <c r="C16" s="33" t="n">
+        <v>150141</v>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>Capital Gains 2025 tab; K4-vanguard-working-2025.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ränteutgifter (Santander UK interest only)</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="n">
+        <v>89876</v>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Santander tab; £6,955 × 12.92163</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Avräkning utländsk skatt</t>
+        </is>
+      </c>
+      <c r="C19" s="53" t="n">
+        <v>5608</v>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>9/12 UK 25/26 (£214) + 3/12 UK 24/25 (£1,092) × 12.92163</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>K4 avsnitt A — Vanguard ISA (4 funds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>Antal</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>Beteckning</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>Försäljningspris (SEK)</t>
+        </is>
+      </c>
+      <c r="D22" s="31" t="inlineStr">
+        <is>
+          <t>Omkostnadsbelopp (SEK)</t>
+        </is>
+      </c>
+      <c r="E22" s="31" t="inlineStr">
+        <is>
+          <t>Vinst (SEK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>74</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>FTSE 100 Index Unit Trust Accumulation</t>
+        </is>
+      </c>
+      <c r="C23" s="33" t="n">
+        <v>173014</v>
+      </c>
+      <c r="D23" s="33" t="n">
+        <v>99683</v>
+      </c>
+      <c r="E23" s="33" t="n">
+        <v>73331</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>155</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>S&amp;P 500 UCITS ETF (VUSA)</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="n">
+        <v>168353</v>
+      </c>
+      <c r="D24" s="33" t="n">
+        <v>98869</v>
+      </c>
+      <c r="E24" s="33" t="n">
+        <v>69484</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>45</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FTSE 250 UCITS ETF (VMID)</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="n">
+        <v>18869</v>
+      </c>
+      <c r="D25" s="33" t="n">
+        <v>17495</v>
+      </c>
+      <c r="E25" s="33" t="n">
+        <v>1374</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>42</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>FTSE Developed Europe ex UK (VERX)</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="n">
+        <v>19957</v>
+      </c>
+      <c r="D26" s="33" t="n">
+        <v>14005</v>
+      </c>
+      <c r="E26" s="33" t="n">
+        <v>5952</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="46" t="n"/>
+      <c r="B27" s="54" t="inlineStr">
+        <is>
+          <t>Summa</t>
+        </is>
+      </c>
+      <c r="C27" s="55" t="n">
+        <v>380193</v>
+      </c>
+      <c r="D27" s="55" t="n">
+        <v>230052</v>
+      </c>
+      <c r="E27" s="55" t="n">
+        <v>150141</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>UK SA100/SA105 2025/26 — submitted values</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>Box</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C30" s="31" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="D30" s="31" t="inlineStr"/>
+      <c r="E30" s="31" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>SA100 TR3 box 2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Untaxed UK interest (HSBC)</t>
+        </is>
+      </c>
+      <c r="C31" s="42" t="n">
+        <v>242</v>
+      </c>
+      <c r="E31" s="16" t="inlineStr">
+        <is>
+          <t>HSBC Interest tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>SA105 box 20</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Total rents received (gross)</t>
+        </is>
+      </c>
+      <c r="C32" s="42" t="n">
+        <v>32271</v>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>76A Ingelow Road tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>SA105 box 25</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Property repairs &amp; maintenance</t>
+        </is>
+      </c>
+      <c r="C33" s="42" t="n">
+        <v>7943</v>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>76A Ingelow Road tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>SA105 box 27</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Legal, management, prof fees</t>
+        </is>
+      </c>
+      <c r="C34" s="42" t="n">
+        <v>2859</v>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>Knight Frank</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>SA105 box 38</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Adjusted profit</t>
+        </is>
+      </c>
+      <c r="C35" s="42" t="n">
+        <v>21469</v>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
+        <is>
+          <t>Tax 25-26 tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>SA105 box 40</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Taxable profit</t>
+        </is>
+      </c>
+      <c r="C36" s="42" t="n">
+        <v>21469</v>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>Tax 25-26 tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>SA105 box 44</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Residential property finance costs</t>
+        </is>
+      </c>
+      <c r="C37" s="42" t="n">
+        <v>7830</v>
+      </c>
+      <c r="E37" s="16" t="inlineStr">
+        <is>
+          <t>Santander tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>SA110 box 1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Total tax due</t>
+        </is>
+      </c>
+      <c r="C38" s="42" t="n">
+        <v>213.8</v>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>Tax 25-26 tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>FX rates used (Riksbanken)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="31" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B41" s="31" t="inlineStr">
+        <is>
+          <t>Rate (SEK/GBP)</t>
+        </is>
+      </c>
+      <c r="C41" s="31" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr"/>
+      <c r="E41" s="31" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sep 2020 – Nov 2021 (monthly Medel)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>11.24–11.98</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Vanguard buys (per Capital Gains 2025 tab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Jun 2025 Medel</t>
+        </is>
+      </c>
+      <c r="B43" s="43" t="n">
+        <v>12.9485</v>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>Vanguard sale (all 4 funds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025 årsmedel</t>
+        </is>
+      </c>
+      <c r="B44" s="43" t="n">
+        <v>12.92163</v>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Recurring items (rental, interest, FTC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="30" t="inlineStr">
+        <is>
+          <t>Companion files (this folder)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="56" t="inlineStr">
+        <is>
+          <t>Tax_Filing_Guide_2025.md</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Canonical post-filing reference (positions + statutory anchors)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="56" t="inlineStr">
+        <is>
+          <t>Tax_Filing_Guide_2025.docx</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Word copy regenerated from .md</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="56" t="inlineStr">
+        <is>
+          <t>K4-vanguard-working-2025.md</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Per-fund Vanguard genomsnittsmetoden detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="56" t="inlineStr">
+        <is>
+          <t>Ovriga_upplysningar_2025.md</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Three blocks for Skatteverket free-text</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="56" t="inlineStr">
+        <is>
+          <t>Swedish_Tax_Return_2025_filed.md</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Submission record incl. all values + kvittens</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="56" t="inlineStr">
+        <is>
+          <t>Swedish_Tax_Return_2025_kvittens.pdf</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Skatteverket receipt PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="56" t="inlineStr">
+        <is>
+          <t>UK_Tax_Return_2025-26_filed.pdf</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>HMRC submission PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="56" t="inlineStr">
+        <is>
+          <t>UK_Tax_Return_2025-26_submission_receipt.pdf</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HMRC receipt PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="56" t="inlineStr">
+        <is>
+          <t>vanguard-transactions/*.pdf</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Vanguard ISA transaction history (evidence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="56" t="inlineStr">
+        <is>
+          <t>Next_Year_Checklist.md</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Roadmap for 2026 returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="56" t="inlineStr">
+        <is>
+          <t>notes.md</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Mortgage history + tax-year totals</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="B49:E49"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="B55:E55"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="B50:E50"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="A46:E46"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="B56:E56"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="B52:E52"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A9:E9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B1:AY16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
@@ -2836,7 +3709,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4422,7 +5295,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5075,7 +5948,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5097,7 +5970,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -5214,7 +6086,6 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
@@ -5288,7 +6159,6 @@
         <v/>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
@@ -5329,7 +6199,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="13" t="inlineStr">
         <is>
@@ -5396,8 +6265,6 @@
         <v/>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
@@ -5466,7 +6333,6 @@
         <v/>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
         <is>
@@ -5519,7 +6385,6 @@
         <v/>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
         <is>
@@ -5531,7 +6396,6 @@
         <v/>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="13" t="inlineStr">
         <is>
@@ -5586,7 +6450,6 @@
         <v/>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
         <is>
@@ -5643,8 +6506,6 @@
         <v/>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
     <row r="59">
       <c r="A59" s="13" t="inlineStr">
         <is>
@@ -5670,7 +6531,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="B63" s="12" t="inlineStr">
         <is>
@@ -5996,7 +6856,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6716,7 +7576,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7347,7 +8207,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7372,7 +8232,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -7401,8 +8260,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="30" t="inlineStr">
         <is>
@@ -7549,7 +8406,6 @@
         <v/>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="30" t="inlineStr">
         <is>

</xml_diff>